<commit_message>
fix modificacion de sp AC_pro_GetClientsEntities
</commit_message>
<xml_diff>
--- a/Guias Produccion/HU-57723.xlsx
+++ b/Guias Produccion/HU-57723.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Alliance\ScriptsEntidades\Guias Produccion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B69ABD94-2576-45C3-B8BE-8F3AF5470FE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5745683B-F80A-4243-BD5C-5903C45993AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Guia de implementación" sheetId="1" r:id="rId1"/>
@@ -1980,95 +1980,8 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="75" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="76" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="77" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="51" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="52" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="54" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="78" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="79" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="60" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="61" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="65" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="62" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="66" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="40" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="55" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="71" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="51" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="52" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="53" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="72" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="73" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="74" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2172,6 +2085,96 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="51" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="52" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="54" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="78" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="79" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="60" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="61" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="65" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="62" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="66" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="40" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="55" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="71" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="51" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="52" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="53" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="72" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="73" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="74" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="10" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2243,9 +2246,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="9" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -11217,42 +11217,42 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:15" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="126" t="s">
+      <c r="A3" s="97" t="s">
         <v>103</v>
       </c>
-      <c r="B3" s="127"/>
-      <c r="C3" s="127"/>
-      <c r="D3" s="127"/>
-      <c r="E3" s="127"/>
-      <c r="F3" s="127"/>
-      <c r="G3" s="127"/>
-      <c r="H3" s="127"/>
-      <c r="I3" s="127"/>
-      <c r="J3" s="127"/>
-      <c r="K3" s="127"/>
-      <c r="L3" s="128"/>
-      <c r="N3" s="120" t="s">
+      <c r="B3" s="98"/>
+      <c r="C3" s="98"/>
+      <c r="D3" s="98"/>
+      <c r="E3" s="98"/>
+      <c r="F3" s="98"/>
+      <c r="G3" s="98"/>
+      <c r="H3" s="98"/>
+      <c r="I3" s="98"/>
+      <c r="J3" s="98"/>
+      <c r="K3" s="98"/>
+      <c r="L3" s="99"/>
+      <c r="N3" s="91" t="s">
         <v>0</v>
       </c>
-      <c r="O3" s="121"/>
+      <c r="O3" s="92"/>
     </row>
     <row r="4" spans="1:15" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="133" t="s">
+      <c r="B4" s="104" t="s">
         <v>105</v>
       </c>
-      <c r="C4" s="134"/>
-      <c r="D4" s="134"/>
-      <c r="E4" s="134"/>
-      <c r="F4" s="134"/>
-      <c r="G4" s="134"/>
-      <c r="H4" s="134"/>
-      <c r="I4" s="134"/>
-      <c r="J4" s="135"/>
-      <c r="K4" s="135"/>
-      <c r="L4" s="136"/>
+      <c r="C4" s="105"/>
+      <c r="D4" s="105"/>
+      <c r="E4" s="105"/>
+      <c r="F4" s="105"/>
+      <c r="G4" s="105"/>
+      <c r="H4" s="105"/>
+      <c r="I4" s="105"/>
+      <c r="J4" s="106"/>
+      <c r="K4" s="106"/>
+      <c r="L4" s="107"/>
       <c r="N4" s="21" t="s">
         <v>2</v>
       </c>
@@ -11262,19 +11262,19 @@
       <c r="A5" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="137" t="s">
+      <c r="B5" s="108" t="s">
         <v>109</v>
       </c>
-      <c r="C5" s="137"/>
-      <c r="D5" s="137"/>
-      <c r="E5" s="137"/>
-      <c r="F5" s="137"/>
-      <c r="G5" s="137"/>
-      <c r="H5" s="137"/>
-      <c r="I5" s="137"/>
-      <c r="J5" s="138"/>
-      <c r="K5" s="138"/>
-      <c r="L5" s="139"/>
+      <c r="C5" s="108"/>
+      <c r="D5" s="108"/>
+      <c r="E5" s="108"/>
+      <c r="F5" s="108"/>
+      <c r="G5" s="108"/>
+      <c r="H5" s="108"/>
+      <c r="I5" s="108"/>
+      <c r="J5" s="109"/>
+      <c r="K5" s="109"/>
+      <c r="L5" s="110"/>
       <c r="N5" s="15" t="s">
         <v>4</v>
       </c>
@@ -11284,19 +11284,19 @@
       <c r="A6" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="123">
+      <c r="B6" s="94">
         <v>46073</v>
       </c>
-      <c r="C6" s="124"/>
-      <c r="D6" s="124"/>
-      <c r="E6" s="124"/>
-      <c r="F6" s="124"/>
-      <c r="G6" s="124"/>
-      <c r="H6" s="124"/>
-      <c r="I6" s="124"/>
-      <c r="J6" s="124"/>
-      <c r="K6" s="124"/>
-      <c r="L6" s="125"/>
+      <c r="C6" s="95"/>
+      <c r="D6" s="95"/>
+      <c r="E6" s="95"/>
+      <c r="F6" s="95"/>
+      <c r="G6" s="95"/>
+      <c r="H6" s="95"/>
+      <c r="I6" s="95"/>
+      <c r="J6" s="95"/>
+      <c r="K6" s="95"/>
+      <c r="L6" s="96"/>
       <c r="N6" s="14"/>
       <c r="O6" s="14"/>
     </row>
@@ -11304,17 +11304,17 @@
       <c r="A7" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="140"/>
-      <c r="C7" s="141"/>
-      <c r="D7" s="141"/>
-      <c r="E7" s="141"/>
-      <c r="F7" s="141"/>
-      <c r="G7" s="141"/>
-      <c r="H7" s="141"/>
-      <c r="I7" s="141"/>
-      <c r="J7" s="142"/>
-      <c r="K7" s="142"/>
-      <c r="L7" s="143"/>
+      <c r="B7" s="111"/>
+      <c r="C7" s="112"/>
+      <c r="D7" s="112"/>
+      <c r="E7" s="112"/>
+      <c r="F7" s="112"/>
+      <c r="G7" s="112"/>
+      <c r="H7" s="112"/>
+      <c r="I7" s="112"/>
+      <c r="J7" s="113"/>
+      <c r="K7" s="113"/>
+      <c r="L7" s="114"/>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" s="11"/>
@@ -11331,20 +11331,20 @@
       <c r="L8" s="13"/>
     </row>
     <row r="9" spans="1:15" s="5" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="129" t="s">
+      <c r="A9" s="100" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="130"/>
-      <c r="C9" s="130"/>
-      <c r="D9" s="130"/>
-      <c r="E9" s="130"/>
-      <c r="F9" s="130"/>
-      <c r="G9" s="130"/>
-      <c r="H9" s="130"/>
-      <c r="I9" s="130"/>
-      <c r="J9" s="131"/>
-      <c r="K9" s="131"/>
-      <c r="L9" s="132"/>
+      <c r="B9" s="101"/>
+      <c r="C9" s="101"/>
+      <c r="D9" s="101"/>
+      <c r="E9" s="101"/>
+      <c r="F9" s="101"/>
+      <c r="G9" s="101"/>
+      <c r="H9" s="101"/>
+      <c r="I9" s="101"/>
+      <c r="J9" s="102"/>
+      <c r="K9" s="102"/>
+      <c r="L9" s="103"/>
     </row>
     <row r="10" spans="1:15" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
@@ -11444,63 +11444,63 @@
       <c r="A14" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="B14" s="122"/>
-      <c r="C14" s="118"/>
-      <c r="D14" s="118"/>
-      <c r="E14" s="118"/>
-      <c r="F14" s="118"/>
-      <c r="G14" s="118"/>
-      <c r="H14" s="118"/>
-      <c r="I14" s="118"/>
-      <c r="J14" s="118"/>
-      <c r="K14" s="118"/>
-      <c r="L14" s="119"/>
+      <c r="B14" s="93"/>
+      <c r="C14" s="89"/>
+      <c r="D14" s="89"/>
+      <c r="E14" s="89"/>
+      <c r="F14" s="89"/>
+      <c r="G14" s="89"/>
+      <c r="H14" s="89"/>
+      <c r="I14" s="89"/>
+      <c r="J14" s="89"/>
+      <c r="K14" s="89"/>
+      <c r="L14" s="90"/>
     </row>
     <row r="15" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="B15" s="117"/>
-      <c r="C15" s="118"/>
-      <c r="D15" s="118"/>
-      <c r="E15" s="118"/>
-      <c r="F15" s="118"/>
-      <c r="G15" s="118"/>
-      <c r="H15" s="118"/>
-      <c r="I15" s="118"/>
-      <c r="J15" s="118"/>
-      <c r="K15" s="118"/>
-      <c r="L15" s="119"/>
+      <c r="B15" s="88"/>
+      <c r="C15" s="89"/>
+      <c r="D15" s="89"/>
+      <c r="E15" s="89"/>
+      <c r="F15" s="89"/>
+      <c r="G15" s="89"/>
+      <c r="H15" s="89"/>
+      <c r="I15" s="89"/>
+      <c r="J15" s="89"/>
+      <c r="K15" s="89"/>
+      <c r="L15" s="90"/>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A16" s="110"/>
-      <c r="B16" s="111"/>
-      <c r="C16" s="111"/>
-      <c r="D16" s="111"/>
-      <c r="E16" s="111"/>
-      <c r="F16" s="111"/>
-      <c r="G16" s="111"/>
-      <c r="H16" s="111"/>
-      <c r="I16" s="111"/>
-      <c r="J16" s="111"/>
-      <c r="K16" s="111"/>
-      <c r="L16" s="112"/>
+      <c r="A16" s="81"/>
+      <c r="B16" s="82"/>
+      <c r="C16" s="82"/>
+      <c r="D16" s="82"/>
+      <c r="E16" s="82"/>
+      <c r="F16" s="82"/>
+      <c r="G16" s="82"/>
+      <c r="H16" s="82"/>
+      <c r="I16" s="82"/>
+      <c r="J16" s="82"/>
+      <c r="K16" s="82"/>
+      <c r="L16" s="83"/>
     </row>
     <row r="17" spans="1:12" s="5" customFormat="1" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="113" t="s">
+      <c r="A17" s="84" t="s">
         <v>25</v>
       </c>
-      <c r="B17" s="114"/>
-      <c r="C17" s="114"/>
-      <c r="D17" s="114"/>
-      <c r="E17" s="114"/>
-      <c r="F17" s="114"/>
-      <c r="G17" s="114"/>
-      <c r="H17" s="114"/>
-      <c r="I17" s="114"/>
-      <c r="J17" s="115"/>
-      <c r="K17" s="115"/>
-      <c r="L17" s="116"/>
+      <c r="B17" s="85"/>
+      <c r="C17" s="85"/>
+      <c r="D17" s="85"/>
+      <c r="E17" s="85"/>
+      <c r="F17" s="85"/>
+      <c r="G17" s="85"/>
+      <c r="H17" s="85"/>
+      <c r="I17" s="85"/>
+      <c r="J17" s="86"/>
+      <c r="K17" s="86"/>
+      <c r="L17" s="87"/>
     </row>
     <row r="18" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="6"/>
@@ -11510,19 +11510,19 @@
       <c r="C18" s="43" t="s">
         <v>27</v>
       </c>
-      <c r="D18" s="86" t="s">
+      <c r="D18" s="121" t="s">
         <v>28</v>
       </c>
-      <c r="E18" s="88" t="s">
+      <c r="E18" s="123" t="s">
         <v>137</v>
       </c>
-      <c r="F18" s="88"/>
-      <c r="G18" s="88"/>
-      <c r="H18" s="88"/>
-      <c r="I18" s="88"/>
-      <c r="J18" s="89"/>
-      <c r="K18" s="89"/>
-      <c r="L18" s="90"/>
+      <c r="F18" s="123"/>
+      <c r="G18" s="123"/>
+      <c r="H18" s="123"/>
+      <c r="I18" s="123"/>
+      <c r="J18" s="124"/>
+      <c r="K18" s="124"/>
+      <c r="L18" s="125"/>
     </row>
     <row r="19" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="8" t="s">
@@ -11532,15 +11532,15 @@
         <v>30</v>
       </c>
       <c r="C19" s="44"/>
-      <c r="D19" s="87"/>
-      <c r="E19" s="91"/>
-      <c r="F19" s="91"/>
-      <c r="G19" s="91"/>
-      <c r="H19" s="91"/>
-      <c r="I19" s="91"/>
-      <c r="J19" s="92"/>
-      <c r="K19" s="92"/>
-      <c r="L19" s="93"/>
+      <c r="D19" s="122"/>
+      <c r="E19" s="126"/>
+      <c r="F19" s="126"/>
+      <c r="G19" s="126"/>
+      <c r="H19" s="126"/>
+      <c r="I19" s="126"/>
+      <c r="J19" s="127"/>
+      <c r="K19" s="127"/>
+      <c r="L19" s="128"/>
     </row>
     <row r="20" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="8" t="s">
@@ -11550,15 +11550,15 @@
       <c r="C20" s="44" t="s">
         <v>30</v>
       </c>
-      <c r="D20" s="87"/>
-      <c r="E20" s="91"/>
-      <c r="F20" s="91"/>
-      <c r="G20" s="91"/>
-      <c r="H20" s="91"/>
-      <c r="I20" s="91"/>
-      <c r="J20" s="92"/>
-      <c r="K20" s="92"/>
-      <c r="L20" s="93"/>
+      <c r="D20" s="122"/>
+      <c r="E20" s="126"/>
+      <c r="F20" s="126"/>
+      <c r="G20" s="126"/>
+      <c r="H20" s="126"/>
+      <c r="I20" s="126"/>
+      <c r="J20" s="127"/>
+      <c r="K20" s="127"/>
+      <c r="L20" s="128"/>
     </row>
     <row r="21" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="8" t="s">
@@ -11568,19 +11568,19 @@
       <c r="C21" s="44" t="s">
         <v>30</v>
       </c>
-      <c r="D21" s="102" t="s">
+      <c r="D21" s="137" t="s">
         <v>25</v>
       </c>
-      <c r="E21" s="104" t="s">
+      <c r="E21" s="139" t="s">
         <v>107</v>
       </c>
-      <c r="F21" s="105"/>
-      <c r="G21" s="105"/>
-      <c r="H21" s="105"/>
-      <c r="I21" s="105"/>
-      <c r="J21" s="105"/>
-      <c r="K21" s="105"/>
-      <c r="L21" s="106"/>
+      <c r="F21" s="140"/>
+      <c r="G21" s="140"/>
+      <c r="H21" s="140"/>
+      <c r="I21" s="140"/>
+      <c r="J21" s="140"/>
+      <c r="K21" s="140"/>
+      <c r="L21" s="141"/>
     </row>
     <row r="22" spans="1:12" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="8" t="s">
@@ -11590,45 +11590,45 @@
       <c r="C22" s="44" t="s">
         <v>30</v>
       </c>
-      <c r="D22" s="103"/>
-      <c r="E22" s="107"/>
-      <c r="F22" s="108"/>
-      <c r="G22" s="108"/>
-      <c r="H22" s="108"/>
-      <c r="I22" s="108"/>
-      <c r="J22" s="108"/>
-      <c r="K22" s="108"/>
-      <c r="L22" s="109"/>
+      <c r="D22" s="138"/>
+      <c r="E22" s="142"/>
+      <c r="F22" s="143"/>
+      <c r="G22" s="143"/>
+      <c r="H22" s="143"/>
+      <c r="I22" s="143"/>
+      <c r="J22" s="143"/>
+      <c r="K22" s="143"/>
+      <c r="L22" s="144"/>
     </row>
     <row r="23" spans="1:12" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="95"/>
-      <c r="B23" s="96"/>
-      <c r="C23" s="96"/>
-      <c r="D23" s="97"/>
-      <c r="E23" s="97"/>
-      <c r="F23" s="97"/>
-      <c r="G23" s="97"/>
-      <c r="H23" s="97"/>
-      <c r="I23" s="97"/>
-      <c r="J23" s="97"/>
-      <c r="K23" s="97"/>
-      <c r="L23" s="98"/>
+      <c r="A23" s="130"/>
+      <c r="B23" s="131"/>
+      <c r="C23" s="131"/>
+      <c r="D23" s="132"/>
+      <c r="E23" s="132"/>
+      <c r="F23" s="132"/>
+      <c r="G23" s="132"/>
+      <c r="H23" s="132"/>
+      <c r="I23" s="132"/>
+      <c r="J23" s="132"/>
+      <c r="K23" s="132"/>
+      <c r="L23" s="133"/>
     </row>
     <row r="24" spans="1:12" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A24" s="99" t="s">
+      <c r="A24" s="134" t="s">
         <v>34</v>
       </c>
-      <c r="B24" s="100"/>
-      <c r="C24" s="100"/>
-      <c r="D24" s="100"/>
-      <c r="E24" s="100"/>
-      <c r="F24" s="100"/>
-      <c r="G24" s="100"/>
-      <c r="H24" s="100"/>
-      <c r="I24" s="100"/>
-      <c r="J24" s="100"/>
-      <c r="K24" s="100"/>
-      <c r="L24" s="101"/>
+      <c r="B24" s="135"/>
+      <c r="C24" s="135"/>
+      <c r="D24" s="135"/>
+      <c r="E24" s="135"/>
+      <c r="F24" s="135"/>
+      <c r="G24" s="135"/>
+      <c r="H24" s="135"/>
+      <c r="I24" s="135"/>
+      <c r="J24" s="135"/>
+      <c r="K24" s="135"/>
+      <c r="L24" s="136"/>
     </row>
     <row r="25" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A25" s="16" t="s">
@@ -11640,17 +11640,17 @@
       <c r="C25" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="D25" s="94" t="s">
+      <c r="D25" s="129" t="s">
         <v>38</v>
       </c>
-      <c r="E25" s="94"/>
-      <c r="F25" s="94"/>
-      <c r="G25" s="94"/>
-      <c r="H25" s="94"/>
-      <c r="I25" s="94"/>
-      <c r="J25" s="94"/>
-      <c r="K25" s="94"/>
-      <c r="L25" s="94"/>
+      <c r="E25" s="129"/>
+      <c r="F25" s="129"/>
+      <c r="G25" s="129"/>
+      <c r="H25" s="129"/>
+      <c r="I25" s="129"/>
+      <c r="J25" s="129"/>
+      <c r="K25" s="129"/>
+      <c r="L25" s="129"/>
     </row>
     <row r="26" spans="1:12" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="33">
@@ -11660,17 +11660,17 @@
         <v>115</v>
       </c>
       <c r="C26" s="34"/>
-      <c r="D26" s="80" t="s">
+      <c r="D26" s="115" t="s">
         <v>108</v>
       </c>
-      <c r="E26" s="81"/>
-      <c r="F26" s="81"/>
-      <c r="G26" s="81"/>
-      <c r="H26" s="81"/>
-      <c r="I26" s="81"/>
-      <c r="J26" s="81"/>
-      <c r="K26" s="81"/>
-      <c r="L26" s="81"/>
+      <c r="E26" s="116"/>
+      <c r="F26" s="116"/>
+      <c r="G26" s="116"/>
+      <c r="H26" s="116"/>
+      <c r="I26" s="116"/>
+      <c r="J26" s="116"/>
+      <c r="K26" s="116"/>
+      <c r="L26" s="116"/>
     </row>
     <row r="27" spans="1:12" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="33">
@@ -11680,15 +11680,15 @@
         <v>116</v>
       </c>
       <c r="C27" s="34"/>
-      <c r="D27" s="82"/>
-      <c r="E27" s="83"/>
-      <c r="F27" s="83"/>
-      <c r="G27" s="83"/>
-      <c r="H27" s="83"/>
-      <c r="I27" s="83"/>
-      <c r="J27" s="83"/>
-      <c r="K27" s="83"/>
-      <c r="L27" s="83"/>
+      <c r="D27" s="117"/>
+      <c r="E27" s="118"/>
+      <c r="F27" s="118"/>
+      <c r="G27" s="118"/>
+      <c r="H27" s="118"/>
+      <c r="I27" s="118"/>
+      <c r="J27" s="118"/>
+      <c r="K27" s="118"/>
+      <c r="L27" s="118"/>
     </row>
     <row r="28" spans="1:12" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="33">
@@ -11698,15 +11698,15 @@
         <v>117</v>
       </c>
       <c r="C28" s="34"/>
-      <c r="D28" s="82"/>
-      <c r="E28" s="83"/>
-      <c r="F28" s="83"/>
-      <c r="G28" s="83"/>
-      <c r="H28" s="83"/>
-      <c r="I28" s="83"/>
-      <c r="J28" s="83"/>
-      <c r="K28" s="83"/>
-      <c r="L28" s="83"/>
+      <c r="D28" s="117"/>
+      <c r="E28" s="118"/>
+      <c r="F28" s="118"/>
+      <c r="G28" s="118"/>
+      <c r="H28" s="118"/>
+      <c r="I28" s="118"/>
+      <c r="J28" s="118"/>
+      <c r="K28" s="118"/>
+      <c r="L28" s="118"/>
     </row>
     <row r="29" spans="1:12" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="33">
@@ -11716,15 +11716,15 @@
         <v>138</v>
       </c>
       <c r="C29" s="34"/>
-      <c r="D29" s="82"/>
-      <c r="E29" s="83"/>
-      <c r="F29" s="83"/>
-      <c r="G29" s="83"/>
-      <c r="H29" s="83"/>
-      <c r="I29" s="83"/>
-      <c r="J29" s="83"/>
-      <c r="K29" s="83"/>
-      <c r="L29" s="83"/>
+      <c r="D29" s="117"/>
+      <c r="E29" s="118"/>
+      <c r="F29" s="118"/>
+      <c r="G29" s="118"/>
+      <c r="H29" s="118"/>
+      <c r="I29" s="118"/>
+      <c r="J29" s="118"/>
+      <c r="K29" s="118"/>
+      <c r="L29" s="118"/>
     </row>
     <row r="30" spans="1:12" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="33">
@@ -11734,15 +11734,15 @@
         <v>118</v>
       </c>
       <c r="C30" s="34"/>
-      <c r="D30" s="82"/>
-      <c r="E30" s="83"/>
-      <c r="F30" s="83"/>
-      <c r="G30" s="83"/>
-      <c r="H30" s="83"/>
-      <c r="I30" s="83"/>
-      <c r="J30" s="83"/>
-      <c r="K30" s="83"/>
-      <c r="L30" s="83"/>
+      <c r="D30" s="117"/>
+      <c r="E30" s="118"/>
+      <c r="F30" s="118"/>
+      <c r="G30" s="118"/>
+      <c r="H30" s="118"/>
+      <c r="I30" s="118"/>
+      <c r="J30" s="118"/>
+      <c r="K30" s="118"/>
+      <c r="L30" s="118"/>
     </row>
     <row r="31" spans="1:12" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="33">
@@ -11752,15 +11752,15 @@
         <v>119</v>
       </c>
       <c r="C31" s="34"/>
-      <c r="D31" s="82"/>
-      <c r="E31" s="83"/>
-      <c r="F31" s="83"/>
-      <c r="G31" s="83"/>
-      <c r="H31" s="83"/>
-      <c r="I31" s="83"/>
-      <c r="J31" s="83"/>
-      <c r="K31" s="83"/>
-      <c r="L31" s="83"/>
+      <c r="D31" s="117"/>
+      <c r="E31" s="118"/>
+      <c r="F31" s="118"/>
+      <c r="G31" s="118"/>
+      <c r="H31" s="118"/>
+      <c r="I31" s="118"/>
+      <c r="J31" s="118"/>
+      <c r="K31" s="118"/>
+      <c r="L31" s="118"/>
     </row>
     <row r="32" spans="1:12" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="33">
@@ -11770,15 +11770,15 @@
         <v>120</v>
       </c>
       <c r="C32" s="34"/>
-      <c r="D32" s="82"/>
-      <c r="E32" s="83"/>
-      <c r="F32" s="83"/>
-      <c r="G32" s="83"/>
-      <c r="H32" s="83"/>
-      <c r="I32" s="83"/>
-      <c r="J32" s="83"/>
-      <c r="K32" s="83"/>
-      <c r="L32" s="83"/>
+      <c r="D32" s="117"/>
+      <c r="E32" s="118"/>
+      <c r="F32" s="118"/>
+      <c r="G32" s="118"/>
+      <c r="H32" s="118"/>
+      <c r="I32" s="118"/>
+      <c r="J32" s="118"/>
+      <c r="K32" s="118"/>
+      <c r="L32" s="118"/>
     </row>
     <row r="33" spans="1:12" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="33">
@@ -11788,15 +11788,15 @@
         <v>121</v>
       </c>
       <c r="C33" s="34"/>
-      <c r="D33" s="82"/>
-      <c r="E33" s="83"/>
-      <c r="F33" s="83"/>
-      <c r="G33" s="83"/>
-      <c r="H33" s="83"/>
-      <c r="I33" s="83"/>
-      <c r="J33" s="83"/>
-      <c r="K33" s="83"/>
-      <c r="L33" s="83"/>
+      <c r="D33" s="117"/>
+      <c r="E33" s="118"/>
+      <c r="F33" s="118"/>
+      <c r="G33" s="118"/>
+      <c r="H33" s="118"/>
+      <c r="I33" s="118"/>
+      <c r="J33" s="118"/>
+      <c r="K33" s="118"/>
+      <c r="L33" s="118"/>
     </row>
     <row r="34" spans="1:12" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="33">
@@ -11806,15 +11806,15 @@
         <v>122</v>
       </c>
       <c r="C34" s="34"/>
-      <c r="D34" s="82"/>
-      <c r="E34" s="83"/>
-      <c r="F34" s="83"/>
-      <c r="G34" s="83"/>
-      <c r="H34" s="83"/>
-      <c r="I34" s="83"/>
-      <c r="J34" s="83"/>
-      <c r="K34" s="83"/>
-      <c r="L34" s="83"/>
+      <c r="D34" s="117"/>
+      <c r="E34" s="118"/>
+      <c r="F34" s="118"/>
+      <c r="G34" s="118"/>
+      <c r="H34" s="118"/>
+      <c r="I34" s="118"/>
+      <c r="J34" s="118"/>
+      <c r="K34" s="118"/>
+      <c r="L34" s="118"/>
     </row>
     <row r="35" spans="1:12" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="33">
@@ -11824,15 +11824,15 @@
         <v>123</v>
       </c>
       <c r="C35" s="34"/>
-      <c r="D35" s="82"/>
-      <c r="E35" s="83"/>
-      <c r="F35" s="83"/>
-      <c r="G35" s="83"/>
-      <c r="H35" s="83"/>
-      <c r="I35" s="83"/>
-      <c r="J35" s="83"/>
-      <c r="K35" s="83"/>
-      <c r="L35" s="83"/>
+      <c r="D35" s="117"/>
+      <c r="E35" s="118"/>
+      <c r="F35" s="118"/>
+      <c r="G35" s="118"/>
+      <c r="H35" s="118"/>
+      <c r="I35" s="118"/>
+      <c r="J35" s="118"/>
+      <c r="K35" s="118"/>
+      <c r="L35" s="118"/>
     </row>
     <row r="36" spans="1:12" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="33">
@@ -11842,15 +11842,15 @@
         <v>124</v>
       </c>
       <c r="C36" s="34"/>
-      <c r="D36" s="82"/>
-      <c r="E36" s="83"/>
-      <c r="F36" s="83"/>
-      <c r="G36" s="83"/>
-      <c r="H36" s="83"/>
-      <c r="I36" s="83"/>
-      <c r="J36" s="83"/>
-      <c r="K36" s="83"/>
-      <c r="L36" s="83"/>
+      <c r="D36" s="117"/>
+      <c r="E36" s="118"/>
+      <c r="F36" s="118"/>
+      <c r="G36" s="118"/>
+      <c r="H36" s="118"/>
+      <c r="I36" s="118"/>
+      <c r="J36" s="118"/>
+      <c r="K36" s="118"/>
+      <c r="L36" s="118"/>
     </row>
     <row r="37" spans="1:12" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="33">
@@ -11860,15 +11860,15 @@
         <v>139</v>
       </c>
       <c r="C37" s="34"/>
-      <c r="D37" s="82"/>
-      <c r="E37" s="83"/>
-      <c r="F37" s="83"/>
-      <c r="G37" s="83"/>
-      <c r="H37" s="83"/>
-      <c r="I37" s="83"/>
-      <c r="J37" s="83"/>
-      <c r="K37" s="83"/>
-      <c r="L37" s="83"/>
+      <c r="D37" s="117"/>
+      <c r="E37" s="118"/>
+      <c r="F37" s="118"/>
+      <c r="G37" s="118"/>
+      <c r="H37" s="118"/>
+      <c r="I37" s="118"/>
+      <c r="J37" s="118"/>
+      <c r="K37" s="118"/>
+      <c r="L37" s="118"/>
     </row>
     <row r="38" spans="1:12" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="33">
@@ -11878,15 +11878,15 @@
         <v>125</v>
       </c>
       <c r="C38" s="34"/>
-      <c r="D38" s="82"/>
-      <c r="E38" s="83"/>
-      <c r="F38" s="83"/>
-      <c r="G38" s="83"/>
-      <c r="H38" s="83"/>
-      <c r="I38" s="83"/>
-      <c r="J38" s="83"/>
-      <c r="K38" s="83"/>
-      <c r="L38" s="83"/>
+      <c r="D38" s="117"/>
+      <c r="E38" s="118"/>
+      <c r="F38" s="118"/>
+      <c r="G38" s="118"/>
+      <c r="H38" s="118"/>
+      <c r="I38" s="118"/>
+      <c r="J38" s="118"/>
+      <c r="K38" s="118"/>
+      <c r="L38" s="118"/>
     </row>
     <row r="39" spans="1:12" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="33">
@@ -11896,15 +11896,15 @@
         <v>126</v>
       </c>
       <c r="C39" s="34"/>
-      <c r="D39" s="82"/>
-      <c r="E39" s="83"/>
-      <c r="F39" s="83"/>
-      <c r="G39" s="83"/>
-      <c r="H39" s="83"/>
-      <c r="I39" s="83"/>
-      <c r="J39" s="83"/>
-      <c r="K39" s="83"/>
-      <c r="L39" s="83"/>
+      <c r="D39" s="117"/>
+      <c r="E39" s="118"/>
+      <c r="F39" s="118"/>
+      <c r="G39" s="118"/>
+      <c r="H39" s="118"/>
+      <c r="I39" s="118"/>
+      <c r="J39" s="118"/>
+      <c r="K39" s="118"/>
+      <c r="L39" s="118"/>
     </row>
     <row r="40" spans="1:12" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="33">
@@ -11914,15 +11914,15 @@
         <v>127</v>
       </c>
       <c r="C40" s="34"/>
-      <c r="D40" s="82"/>
-      <c r="E40" s="83"/>
-      <c r="F40" s="83"/>
-      <c r="G40" s="83"/>
-      <c r="H40" s="83"/>
-      <c r="I40" s="83"/>
-      <c r="J40" s="83"/>
-      <c r="K40" s="83"/>
-      <c r="L40" s="83"/>
+      <c r="D40" s="117"/>
+      <c r="E40" s="118"/>
+      <c r="F40" s="118"/>
+      <c r="G40" s="118"/>
+      <c r="H40" s="118"/>
+      <c r="I40" s="118"/>
+      <c r="J40" s="118"/>
+      <c r="K40" s="118"/>
+      <c r="L40" s="118"/>
     </row>
     <row r="41" spans="1:12" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="33">
@@ -11932,15 +11932,15 @@
         <v>128</v>
       </c>
       <c r="C41" s="34"/>
-      <c r="D41" s="82"/>
-      <c r="E41" s="83"/>
-      <c r="F41" s="83"/>
-      <c r="G41" s="83"/>
-      <c r="H41" s="83"/>
-      <c r="I41" s="83"/>
-      <c r="J41" s="83"/>
-      <c r="K41" s="83"/>
-      <c r="L41" s="83"/>
+      <c r="D41" s="117"/>
+      <c r="E41" s="118"/>
+      <c r="F41" s="118"/>
+      <c r="G41" s="118"/>
+      <c r="H41" s="118"/>
+      <c r="I41" s="118"/>
+      <c r="J41" s="118"/>
+      <c r="K41" s="118"/>
+      <c r="L41" s="118"/>
     </row>
     <row r="42" spans="1:12" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="33">
@@ -11950,15 +11950,15 @@
         <v>140</v>
       </c>
       <c r="C42" s="34"/>
-      <c r="D42" s="82"/>
-      <c r="E42" s="83"/>
-      <c r="F42" s="83"/>
-      <c r="G42" s="83"/>
-      <c r="H42" s="83"/>
-      <c r="I42" s="83"/>
-      <c r="J42" s="83"/>
-      <c r="K42" s="83"/>
-      <c r="L42" s="83"/>
+      <c r="D42" s="117"/>
+      <c r="E42" s="118"/>
+      <c r="F42" s="118"/>
+      <c r="G42" s="118"/>
+      <c r="H42" s="118"/>
+      <c r="I42" s="118"/>
+      <c r="J42" s="118"/>
+      <c r="K42" s="118"/>
+      <c r="L42" s="118"/>
     </row>
     <row r="43" spans="1:12" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="33">
@@ -11968,15 +11968,15 @@
         <v>141</v>
       </c>
       <c r="C43" s="34"/>
-      <c r="D43" s="82"/>
-      <c r="E43" s="83"/>
-      <c r="F43" s="83"/>
-      <c r="G43" s="83"/>
-      <c r="H43" s="83"/>
-      <c r="I43" s="83"/>
-      <c r="J43" s="83"/>
-      <c r="K43" s="83"/>
-      <c r="L43" s="83"/>
+      <c r="D43" s="117"/>
+      <c r="E43" s="118"/>
+      <c r="F43" s="118"/>
+      <c r="G43" s="118"/>
+      <c r="H43" s="118"/>
+      <c r="I43" s="118"/>
+      <c r="J43" s="118"/>
+      <c r="K43" s="118"/>
+      <c r="L43" s="118"/>
     </row>
     <row r="44" spans="1:12" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="33">
@@ -11986,15 +11986,15 @@
         <v>129</v>
       </c>
       <c r="C44" s="34"/>
-      <c r="D44" s="82"/>
-      <c r="E44" s="83"/>
-      <c r="F44" s="83"/>
-      <c r="G44" s="83"/>
-      <c r="H44" s="83"/>
-      <c r="I44" s="83"/>
-      <c r="J44" s="83"/>
-      <c r="K44" s="83"/>
-      <c r="L44" s="83"/>
+      <c r="D44" s="117"/>
+      <c r="E44" s="118"/>
+      <c r="F44" s="118"/>
+      <c r="G44" s="118"/>
+      <c r="H44" s="118"/>
+      <c r="I44" s="118"/>
+      <c r="J44" s="118"/>
+      <c r="K44" s="118"/>
+      <c r="L44" s="118"/>
     </row>
     <row r="45" spans="1:12" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="33">
@@ -12004,15 +12004,15 @@
         <v>130</v>
       </c>
       <c r="C45" s="34"/>
-      <c r="D45" s="82"/>
-      <c r="E45" s="83"/>
-      <c r="F45" s="83"/>
-      <c r="G45" s="83"/>
-      <c r="H45" s="83"/>
-      <c r="I45" s="83"/>
-      <c r="J45" s="83"/>
-      <c r="K45" s="83"/>
-      <c r="L45" s="83"/>
+      <c r="D45" s="117"/>
+      <c r="E45" s="118"/>
+      <c r="F45" s="118"/>
+      <c r="G45" s="118"/>
+      <c r="H45" s="118"/>
+      <c r="I45" s="118"/>
+      <c r="J45" s="118"/>
+      <c r="K45" s="118"/>
+      <c r="L45" s="118"/>
     </row>
     <row r="46" spans="1:12" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="33">
@@ -12022,15 +12022,15 @@
         <v>131</v>
       </c>
       <c r="C46" s="34"/>
-      <c r="D46" s="82"/>
-      <c r="E46" s="83"/>
-      <c r="F46" s="83"/>
-      <c r="G46" s="83"/>
-      <c r="H46" s="83"/>
-      <c r="I46" s="83"/>
-      <c r="J46" s="83"/>
-      <c r="K46" s="83"/>
-      <c r="L46" s="83"/>
+      <c r="D46" s="117"/>
+      <c r="E46" s="118"/>
+      <c r="F46" s="118"/>
+      <c r="G46" s="118"/>
+      <c r="H46" s="118"/>
+      <c r="I46" s="118"/>
+      <c r="J46" s="118"/>
+      <c r="K46" s="118"/>
+      <c r="L46" s="118"/>
     </row>
     <row r="47" spans="1:12" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="33">
@@ -12040,15 +12040,15 @@
         <v>132</v>
       </c>
       <c r="C47" s="34"/>
-      <c r="D47" s="82"/>
-      <c r="E47" s="83"/>
-      <c r="F47" s="83"/>
-      <c r="G47" s="83"/>
-      <c r="H47" s="83"/>
-      <c r="I47" s="83"/>
-      <c r="J47" s="83"/>
-      <c r="K47" s="83"/>
-      <c r="L47" s="83"/>
+      <c r="D47" s="117"/>
+      <c r="E47" s="118"/>
+      <c r="F47" s="118"/>
+      <c r="G47" s="118"/>
+      <c r="H47" s="118"/>
+      <c r="I47" s="118"/>
+      <c r="J47" s="118"/>
+      <c r="K47" s="118"/>
+      <c r="L47" s="118"/>
     </row>
     <row r="48" spans="1:12" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="33">
@@ -12058,15 +12058,15 @@
         <v>133</v>
       </c>
       <c r="C48" s="34"/>
-      <c r="D48" s="82"/>
-      <c r="E48" s="83"/>
-      <c r="F48" s="83"/>
-      <c r="G48" s="83"/>
-      <c r="H48" s="83"/>
-      <c r="I48" s="83"/>
-      <c r="J48" s="83"/>
-      <c r="K48" s="83"/>
-      <c r="L48" s="83"/>
+      <c r="D48" s="117"/>
+      <c r="E48" s="118"/>
+      <c r="F48" s="118"/>
+      <c r="G48" s="118"/>
+      <c r="H48" s="118"/>
+      <c r="I48" s="118"/>
+      <c r="J48" s="118"/>
+      <c r="K48" s="118"/>
+      <c r="L48" s="118"/>
     </row>
     <row r="49" spans="1:12" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="33">
@@ -12076,15 +12076,15 @@
         <v>143</v>
       </c>
       <c r="C49" s="34"/>
-      <c r="D49" s="82"/>
-      <c r="E49" s="83"/>
-      <c r="F49" s="83"/>
-      <c r="G49" s="83"/>
-      <c r="H49" s="83"/>
-      <c r="I49" s="83"/>
-      <c r="J49" s="83"/>
-      <c r="K49" s="83"/>
-      <c r="L49" s="83"/>
+      <c r="D49" s="117"/>
+      <c r="E49" s="118"/>
+      <c r="F49" s="118"/>
+      <c r="G49" s="118"/>
+      <c r="H49" s="118"/>
+      <c r="I49" s="118"/>
+      <c r="J49" s="118"/>
+      <c r="K49" s="118"/>
+      <c r="L49" s="118"/>
     </row>
     <row r="50" spans="1:12" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="72">
@@ -12094,15 +12094,15 @@
         <v>134</v>
       </c>
       <c r="C50" s="34"/>
-      <c r="D50" s="82"/>
-      <c r="E50" s="83"/>
-      <c r="F50" s="83"/>
-      <c r="G50" s="83"/>
-      <c r="H50" s="83"/>
-      <c r="I50" s="83"/>
-      <c r="J50" s="83"/>
-      <c r="K50" s="83"/>
-      <c r="L50" s="83"/>
+      <c r="D50" s="117"/>
+      <c r="E50" s="118"/>
+      <c r="F50" s="118"/>
+      <c r="G50" s="118"/>
+      <c r="H50" s="118"/>
+      <c r="I50" s="118"/>
+      <c r="J50" s="118"/>
+      <c r="K50" s="118"/>
+      <c r="L50" s="118"/>
     </row>
     <row r="51" spans="1:12" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="72">
@@ -12112,15 +12112,15 @@
         <v>135</v>
       </c>
       <c r="C51" s="34"/>
-      <c r="D51" s="82"/>
-      <c r="E51" s="83"/>
-      <c r="F51" s="83"/>
-      <c r="G51" s="83"/>
-      <c r="H51" s="83"/>
-      <c r="I51" s="83"/>
-      <c r="J51" s="83"/>
-      <c r="K51" s="83"/>
-      <c r="L51" s="83"/>
+      <c r="D51" s="117"/>
+      <c r="E51" s="118"/>
+      <c r="F51" s="118"/>
+      <c r="G51" s="118"/>
+      <c r="H51" s="118"/>
+      <c r="I51" s="118"/>
+      <c r="J51" s="118"/>
+      <c r="K51" s="118"/>
+      <c r="L51" s="118"/>
     </row>
     <row r="52" spans="1:12" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="72">
@@ -12130,15 +12130,15 @@
         <v>136</v>
       </c>
       <c r="C52" s="34"/>
-      <c r="D52" s="82"/>
-      <c r="E52" s="83"/>
-      <c r="F52" s="83"/>
-      <c r="G52" s="83"/>
-      <c r="H52" s="83"/>
-      <c r="I52" s="83"/>
-      <c r="J52" s="83"/>
-      <c r="K52" s="83"/>
-      <c r="L52" s="83"/>
+      <c r="D52" s="117"/>
+      <c r="E52" s="118"/>
+      <c r="F52" s="118"/>
+      <c r="G52" s="118"/>
+      <c r="H52" s="118"/>
+      <c r="I52" s="118"/>
+      <c r="J52" s="118"/>
+      <c r="K52" s="118"/>
+      <c r="L52" s="118"/>
     </row>
     <row r="53" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="72">
@@ -12148,15 +12148,15 @@
         <v>142</v>
       </c>
       <c r="C53" s="79"/>
-      <c r="D53" s="82"/>
-      <c r="E53" s="83"/>
-      <c r="F53" s="83"/>
-      <c r="G53" s="83"/>
-      <c r="H53" s="83"/>
-      <c r="I53" s="83"/>
-      <c r="J53" s="83"/>
-      <c r="K53" s="83"/>
-      <c r="L53" s="83"/>
+      <c r="D53" s="117"/>
+      <c r="E53" s="118"/>
+      <c r="F53" s="118"/>
+      <c r="G53" s="118"/>
+      <c r="H53" s="118"/>
+      <c r="I53" s="118"/>
+      <c r="J53" s="118"/>
+      <c r="K53" s="118"/>
+      <c r="L53" s="118"/>
     </row>
     <row r="54" spans="1:12" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="72">
@@ -12166,18 +12166,26 @@
         <v>144</v>
       </c>
       <c r="C54" s="72"/>
-      <c r="D54" s="84"/>
-      <c r="E54" s="85"/>
-      <c r="F54" s="85"/>
-      <c r="G54" s="85"/>
-      <c r="H54" s="85"/>
-      <c r="I54" s="85"/>
-      <c r="J54" s="85"/>
-      <c r="K54" s="85"/>
-      <c r="L54" s="85"/>
+      <c r="D54" s="119"/>
+      <c r="E54" s="120"/>
+      <c r="F54" s="120"/>
+      <c r="G54" s="120"/>
+      <c r="H54" s="120"/>
+      <c r="I54" s="120"/>
+      <c r="J54" s="120"/>
+      <c r="K54" s="120"/>
+      <c r="L54" s="120"/>
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="D26:L54"/>
+    <mergeCell ref="D18:D20"/>
+    <mergeCell ref="E18:L20"/>
+    <mergeCell ref="D25:L25"/>
+    <mergeCell ref="A23:L23"/>
+    <mergeCell ref="A24:L24"/>
+    <mergeCell ref="D21:D22"/>
+    <mergeCell ref="E21:L22"/>
     <mergeCell ref="A16:L16"/>
     <mergeCell ref="A17:L17"/>
     <mergeCell ref="B15:L15"/>
@@ -12189,14 +12197,6 @@
     <mergeCell ref="B4:L4"/>
     <mergeCell ref="B5:L5"/>
     <mergeCell ref="B7:L7"/>
-    <mergeCell ref="D26:L54"/>
-    <mergeCell ref="D18:D20"/>
-    <mergeCell ref="E18:L20"/>
-    <mergeCell ref="D25:L25"/>
-    <mergeCell ref="A23:L23"/>
-    <mergeCell ref="A24:L24"/>
-    <mergeCell ref="D21:D22"/>
-    <mergeCell ref="E21:L22"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="D26" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
@@ -15179,50 +15179,50 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="23.4" x14ac:dyDescent="0.3">
-      <c r="A1" s="153" t="s">
+      <c r="A1" s="154" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="154"/>
-      <c r="C1" s="154"/>
-      <c r="D1" s="154"/>
-      <c r="E1" s="154"/>
-      <c r="F1" s="154"/>
-      <c r="G1" s="154"/>
-      <c r="H1" s="154"/>
-      <c r="I1" s="154"/>
-      <c r="J1" s="154"/>
-      <c r="K1" s="154"/>
-      <c r="L1" s="155"/>
+      <c r="B1" s="155"/>
+      <c r="C1" s="155"/>
+      <c r="D1" s="155"/>
+      <c r="E1" s="155"/>
+      <c r="F1" s="155"/>
+      <c r="G1" s="155"/>
+      <c r="H1" s="155"/>
+      <c r="I1" s="155"/>
+      <c r="J1" s="155"/>
+      <c r="K1" s="155"/>
+      <c r="L1" s="156"/>
     </row>
     <row r="2" spans="1:12" ht="24" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="156" t="s">
+      <c r="A2" s="157" t="s">
         <v>40</v>
       </c>
-      <c r="B2" s="157"/>
-      <c r="C2" s="157"/>
-      <c r="D2" s="157"/>
-      <c r="E2" s="157"/>
-      <c r="F2" s="157"/>
-      <c r="G2" s="157"/>
-      <c r="H2" s="157"/>
-      <c r="I2" s="157"/>
-      <c r="J2" s="157"/>
-      <c r="K2" s="157"/>
-      <c r="L2" s="158"/>
+      <c r="B2" s="158"/>
+      <c r="C2" s="158"/>
+      <c r="D2" s="158"/>
+      <c r="E2" s="158"/>
+      <c r="F2" s="158"/>
+      <c r="G2" s="158"/>
+      <c r="H2" s="158"/>
+      <c r="I2" s="158"/>
+      <c r="J2" s="158"/>
+      <c r="K2" s="158"/>
+      <c r="L2" s="159"/>
     </row>
     <row r="3" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="159"/>
-      <c r="B3" s="160"/>
-      <c r="C3" s="160"/>
-      <c r="D3" s="160"/>
-      <c r="E3" s="160"/>
-      <c r="F3" s="160"/>
-      <c r="G3" s="160"/>
-      <c r="H3" s="160"/>
-      <c r="I3" s="160"/>
-      <c r="J3" s="160"/>
-      <c r="K3" s="160"/>
-      <c r="L3" s="161"/>
+      <c r="A3" s="160"/>
+      <c r="B3" s="161"/>
+      <c r="C3" s="161"/>
+      <c r="D3" s="161"/>
+      <c r="E3" s="161"/>
+      <c r="F3" s="161"/>
+      <c r="G3" s="161"/>
+      <c r="H3" s="161"/>
+      <c r="I3" s="161"/>
+      <c r="J3" s="161"/>
+      <c r="K3" s="161"/>
+      <c r="L3" s="162"/>
     </row>
     <row r="4" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A4" s="2"/>
@@ -15312,65 +15312,65 @@
       <c r="A8" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="B8" s="164"/>
-      <c r="C8" s="165"/>
-      <c r="D8" s="165"/>
-      <c r="E8" s="165"/>
-      <c r="F8" s="165"/>
-      <c r="G8" s="165"/>
-      <c r="H8" s="165"/>
-      <c r="I8" s="165"/>
-      <c r="J8" s="165"/>
-      <c r="K8" s="165"/>
-      <c r="L8" s="166"/>
+      <c r="B8" s="165"/>
+      <c r="C8" s="166"/>
+      <c r="D8" s="166"/>
+      <c r="E8" s="166"/>
+      <c r="F8" s="166"/>
+      <c r="G8" s="166"/>
+      <c r="H8" s="166"/>
+      <c r="I8" s="166"/>
+      <c r="J8" s="166"/>
+      <c r="K8" s="166"/>
+      <c r="L8" s="167"/>
     </row>
     <row r="9" spans="1:12" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="B9" s="167"/>
-      <c r="C9" s="165"/>
-      <c r="D9" s="165"/>
-      <c r="E9" s="165"/>
-      <c r="F9" s="165"/>
-      <c r="G9" s="165"/>
-      <c r="H9" s="165"/>
-      <c r="I9" s="165"/>
-      <c r="J9" s="165"/>
-      <c r="K9" s="165"/>
-      <c r="L9" s="166"/>
+      <c r="B9" s="168"/>
+      <c r="C9" s="166"/>
+      <c r="D9" s="166"/>
+      <c r="E9" s="166"/>
+      <c r="F9" s="166"/>
+      <c r="G9" s="166"/>
+      <c r="H9" s="166"/>
+      <c r="I9" s="166"/>
+      <c r="J9" s="166"/>
+      <c r="K9" s="166"/>
+      <c r="L9" s="167"/>
     </row>
     <row r="10" spans="1:12" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="162" t="s">
+      <c r="A10" s="163" t="s">
         <v>41</v>
       </c>
-      <c r="B10" s="163"/>
-      <c r="C10" s="163"/>
-      <c r="D10" s="163"/>
-      <c r="E10" s="163"/>
-      <c r="F10" s="163"/>
-      <c r="G10" s="163"/>
-      <c r="H10" s="163"/>
-      <c r="I10" s="163"/>
-      <c r="J10" s="163"/>
-      <c r="K10" s="163"/>
-      <c r="L10" s="163"/>
+      <c r="B10" s="164"/>
+      <c r="C10" s="164"/>
+      <c r="D10" s="164"/>
+      <c r="E10" s="164"/>
+      <c r="F10" s="164"/>
+      <c r="G10" s="164"/>
+      <c r="H10" s="164"/>
+      <c r="I10" s="164"/>
+      <c r="J10" s="164"/>
+      <c r="K10" s="164"/>
+      <c r="L10" s="164"/>
     </row>
     <row r="11" spans="1:12" ht="24" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="144" t="s">
+      <c r="A11" s="145" t="s">
         <v>34</v>
       </c>
-      <c r="B11" s="145"/>
-      <c r="C11" s="145"/>
-      <c r="D11" s="145"/>
-      <c r="E11" s="145"/>
-      <c r="F11" s="145"/>
-      <c r="G11" s="145"/>
-      <c r="H11" s="145"/>
-      <c r="I11" s="145"/>
-      <c r="J11" s="145"/>
-      <c r="K11" s="145"/>
-      <c r="L11" s="146"/>
+      <c r="B11" s="146"/>
+      <c r="C11" s="146"/>
+      <c r="D11" s="146"/>
+      <c r="E11" s="146"/>
+      <c r="F11" s="146"/>
+      <c r="G11" s="146"/>
+      <c r="H11" s="146"/>
+      <c r="I11" s="146"/>
+      <c r="J11" s="146"/>
+      <c r="K11" s="146"/>
+      <c r="L11" s="147"/>
     </row>
     <row r="12" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A12" s="16" t="s">
@@ -15382,101 +15382,101 @@
       <c r="C12" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="D12" s="94" t="s">
+      <c r="D12" s="129" t="s">
         <v>38</v>
       </c>
-      <c r="E12" s="94"/>
-      <c r="F12" s="94"/>
-      <c r="G12" s="94"/>
-      <c r="H12" s="94"/>
-      <c r="I12" s="94"/>
-      <c r="J12" s="94"/>
-      <c r="K12" s="94"/>
-      <c r="L12" s="94"/>
+      <c r="E12" s="129"/>
+      <c r="F12" s="129"/>
+      <c r="G12" s="129"/>
+      <c r="H12" s="129"/>
+      <c r="I12" s="129"/>
+      <c r="J12" s="129"/>
+      <c r="K12" s="129"/>
+      <c r="L12" s="129"/>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13" s="49"/>
       <c r="B13" s="50"/>
       <c r="C13" s="50"/>
-      <c r="D13" s="147"/>
-      <c r="E13" s="148"/>
-      <c r="F13" s="148"/>
-      <c r="G13" s="148"/>
-      <c r="H13" s="148"/>
-      <c r="I13" s="148"/>
-      <c r="J13" s="148"/>
-      <c r="K13" s="148"/>
-      <c r="L13" s="149"/>
+      <c r="D13" s="148"/>
+      <c r="E13" s="149"/>
+      <c r="F13" s="149"/>
+      <c r="G13" s="149"/>
+      <c r="H13" s="149"/>
+      <c r="I13" s="149"/>
+      <c r="J13" s="149"/>
+      <c r="K13" s="149"/>
+      <c r="L13" s="150"/>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14" s="49"/>
       <c r="B14" s="50"/>
       <c r="C14" s="50"/>
-      <c r="D14" s="150"/>
-      <c r="E14" s="151"/>
-      <c r="F14" s="151"/>
-      <c r="G14" s="151"/>
-      <c r="H14" s="151"/>
-      <c r="I14" s="151"/>
-      <c r="J14" s="151"/>
-      <c r="K14" s="151"/>
-      <c r="L14" s="152"/>
+      <c r="D14" s="151"/>
+      <c r="E14" s="152"/>
+      <c r="F14" s="152"/>
+      <c r="G14" s="152"/>
+      <c r="H14" s="152"/>
+      <c r="I14" s="152"/>
+      <c r="J14" s="152"/>
+      <c r="K14" s="152"/>
+      <c r="L14" s="153"/>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15" s="49"/>
       <c r="B15" s="50"/>
       <c r="C15" s="50"/>
-      <c r="D15" s="150"/>
-      <c r="E15" s="151"/>
-      <c r="F15" s="151"/>
-      <c r="G15" s="151"/>
-      <c r="H15" s="151"/>
-      <c r="I15" s="151"/>
-      <c r="J15" s="151"/>
-      <c r="K15" s="151"/>
-      <c r="L15" s="152"/>
+      <c r="D15" s="151"/>
+      <c r="E15" s="152"/>
+      <c r="F15" s="152"/>
+      <c r="G15" s="152"/>
+      <c r="H15" s="152"/>
+      <c r="I15" s="152"/>
+      <c r="J15" s="152"/>
+      <c r="K15" s="152"/>
+      <c r="L15" s="153"/>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A16" s="49"/>
       <c r="B16" s="50"/>
       <c r="C16" s="50"/>
-      <c r="D16" s="150"/>
-      <c r="E16" s="151"/>
-      <c r="F16" s="151"/>
-      <c r="G16" s="151"/>
-      <c r="H16" s="151"/>
-      <c r="I16" s="151"/>
-      <c r="J16" s="151"/>
-      <c r="K16" s="151"/>
-      <c r="L16" s="152"/>
+      <c r="D16" s="151"/>
+      <c r="E16" s="152"/>
+      <c r="F16" s="152"/>
+      <c r="G16" s="152"/>
+      <c r="H16" s="152"/>
+      <c r="I16" s="152"/>
+      <c r="J16" s="152"/>
+      <c r="K16" s="152"/>
+      <c r="L16" s="153"/>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A17" s="49"/>
       <c r="B17" s="50"/>
       <c r="C17" s="50"/>
-      <c r="D17" s="150"/>
-      <c r="E17" s="151"/>
-      <c r="F17" s="151"/>
-      <c r="G17" s="151"/>
-      <c r="H17" s="151"/>
-      <c r="I17" s="151"/>
-      <c r="J17" s="151"/>
-      <c r="K17" s="151"/>
-      <c r="L17" s="152"/>
+      <c r="D17" s="151"/>
+      <c r="E17" s="152"/>
+      <c r="F17" s="152"/>
+      <c r="G17" s="152"/>
+      <c r="H17" s="152"/>
+      <c r="I17" s="152"/>
+      <c r="J17" s="152"/>
+      <c r="K17" s="152"/>
+      <c r="L17" s="153"/>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A18" s="49"/>
       <c r="B18" s="50"/>
       <c r="C18" s="50"/>
-      <c r="D18" s="150"/>
-      <c r="E18" s="151"/>
-      <c r="F18" s="151"/>
-      <c r="G18" s="151"/>
-      <c r="H18" s="151"/>
-      <c r="I18" s="151"/>
-      <c r="J18" s="151"/>
-      <c r="K18" s="151"/>
-      <c r="L18" s="152"/>
+      <c r="D18" s="151"/>
+      <c r="E18" s="152"/>
+      <c r="F18" s="152"/>
+      <c r="G18" s="152"/>
+      <c r="H18" s="152"/>
+      <c r="I18" s="152"/>
+      <c r="J18" s="152"/>
+      <c r="K18" s="152"/>
+      <c r="L18" s="153"/>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -15565,10 +15565,10 @@
       <c r="B4" s="63"/>
     </row>
     <row r="6" spans="1:12" ht="18" x14ac:dyDescent="0.35">
-      <c r="A6" s="168" t="s">
+      <c r="A6" s="80" t="s">
         <v>42</v>
       </c>
-      <c r="B6" s="168"/>
+      <c r="B6" s="80"/>
     </row>
     <row r="8" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="66" t="s">
@@ -16300,68 +16300,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <SharedWithUsers xmlns="8029d101-3d2a-47c4-b15f-619642bf5e50">
-      <UserInfo>
-        <DisplayName>Luis Campos / Logiztik Alliance</DisplayName>
-        <AccountId>265</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Jairo Gonzalez / Logiztik Alliance</DisplayName>
-        <AccountId>322</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>José Ganchozo / Logiztik Alliance</DisplayName>
-        <AccountId>304</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Edwin Casa / Logiztik Alliance</DisplayName>
-        <AccountId>299</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Cristhian Cuichan / Logiztik Alliance</DisplayName>
-        <AccountId>369</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Oscar Yunda /  Logiztik Alliance</DisplayName>
-        <AccountId>355</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Fernando Ordoñez / Logiztik Alliance</DisplayName>
-        <AccountId>321</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Alex Rivera / Logiztik Alliance</DisplayName>
-        <AccountId>370</AccountId>
-        <AccountType/>
-      </UserInfo>
-    </SharedWithUsers>
-    <TaxCatchAll xmlns="8029d101-3d2a-47c4-b15f-619642bf5e50" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87481c51-c14c-4071-bf64-faa2b5708bb6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101005DA7AC6E4F4FAE42B9D9FCD9C82CAAE1" ma:contentTypeVersion="17" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="553e0bb76796fbad2df2b84fb95dc83d">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87481c51-c14c-4071-bf64-faa2b5708bb6" xmlns:ns3="8029d101-3d2a-47c4-b15f-619642bf5e50" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d87cd7f238c73dc12c577d08dde48736" ns2:_="" ns3:_="">
     <xsd:import namespace="87481c51-c14c-4071-bf64-faa2b5708bb6"/>
@@ -16610,26 +16548,69 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DD069904-634F-48DA-AA92-BAE250498BEE}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="8029d101-3d2a-47c4-b15f-619642bf5e50"/>
-    <ds:schemaRef ds:uri="87481c51-c14c-4071-bf64-faa2b5708bb6"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{371D8832-41B3-447B-B13D-2663C267E34F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <SharedWithUsers xmlns="8029d101-3d2a-47c4-b15f-619642bf5e50">
+      <UserInfo>
+        <DisplayName>Luis Campos / Logiztik Alliance</DisplayName>
+        <AccountId>265</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Jairo Gonzalez / Logiztik Alliance</DisplayName>
+        <AccountId>322</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>José Ganchozo / Logiztik Alliance</DisplayName>
+        <AccountId>304</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Edwin Casa / Logiztik Alliance</DisplayName>
+        <AccountId>299</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Cristhian Cuichan / Logiztik Alliance</DisplayName>
+        <AccountId>369</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Oscar Yunda /  Logiztik Alliance</DisplayName>
+        <AccountId>355</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Fernando Ordoñez / Logiztik Alliance</DisplayName>
+        <AccountId>321</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Alex Rivera / Logiztik Alliance</DisplayName>
+        <AccountId>370</AccountId>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
+    <TaxCatchAll xmlns="8029d101-3d2a-47c4-b15f-619642bf5e50" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87481c51-c14c-4071-bf64-faa2b5708bb6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2F7F06D0-41B3-4EAF-B418-88FC726117CC}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -16646,4 +16627,23 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{371D8832-41B3-447B-B13D-2663C267E34F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DD069904-634F-48DA-AA92-BAE250498BEE}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="8029d101-3d2a-47c4-b15f-619642bf5e50"/>
+    <ds:schemaRef ds:uri="87481c51-c14c-4071-bf64-faa2b5708bb6"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
fix modificacion de ordenamiento
</commit_message>
<xml_diff>
--- a/Guias Produccion/HU-57723.xlsx
+++ b/Guias Produccion/HU-57723.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Alliance\ScriptsEntidades\Guias Produccion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FCEDC94-5C0C-4DBC-909E-C27EDFC18D3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C0C0A8B-CDE1-4CBF-902C-EB20E9B41D1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="149">
   <si>
     <t>Guia documentación</t>
   </si>
@@ -510,103 +510,106 @@
     <t>Patricia Chicaiza</t>
   </si>
   <si>
-    <t>01-trgUpdateEntityTypes.sql</t>
-  </si>
-  <si>
-    <t>02-trgUpdateEntities.sql</t>
-  </si>
-  <si>
-    <t>03-f_SearchEntities.sql</t>
-  </si>
-  <si>
-    <t>05-AC_pro_GetMachineShipments.sql</t>
-  </si>
-  <si>
-    <t>06-AC_pro_GetClientsPiecesDetails.sql</t>
-  </si>
-  <si>
-    <t>07-AC_pro_GetDispatchesByCarrier.sql</t>
-  </si>
-  <si>
-    <t>08-AC_pro_GetClientsEntities.sql</t>
-  </si>
-  <si>
-    <t>09-AC_pro_GetClientsPiecesBySubCarrier.sql</t>
-  </si>
-  <si>
-    <t>10-AC_pro_GetDispatchesByClient.sql</t>
-  </si>
-  <si>
-    <t>11-AC_pro_GetLocalOrdersByEmployee.sql</t>
-  </si>
-  <si>
-    <t>13-AC_pro_ListCarrierProgramming.sql</t>
-  </si>
-  <si>
-    <t>14-AC_pro_ConfirmLocalOrderCoordination.sql</t>
-  </si>
-  <si>
-    <t>15-AC_pro_ConfirmLocalOrder.sql</t>
-  </si>
-  <si>
-    <t>16-AC_pro_ShippingDocumentsPODClient360.sql</t>
-  </si>
-  <si>
-    <t>19-AC_pro_ListPiecesInventory.sql</t>
-  </si>
-  <si>
-    <t>20-AC_pro_GetBarCodeLinks.sql</t>
-  </si>
-  <si>
-    <t>21-AC_pro_LargeLabelTempDefault.sql</t>
-  </si>
-  <si>
-    <t>22-AC_pro_GetDispatchReports.sql</t>
-  </si>
-  <si>
-    <t>23-AC_pro_GetShipmentAnalyticsReports.sql</t>
-  </si>
-  <si>
-    <t>25-AC_pro_GetCycleCountDiscrepancies.sql</t>
-  </si>
-  <si>
-    <t>26-AC_pro_CycleCountDiscrepanciesReport.sql</t>
-  </si>
-  <si>
-    <t>27-AC_pro_GetConsolidatedDispatchAnalytics.sql</t>
-  </si>
-  <si>
     <t>Es necesario que se ejecuten primero los scripts de la Hu 55188, ya que existe dependencia de algunos campos</t>
   </si>
   <si>
-    <t>04-AC_pro_General_GenerateBulkInt.sql</t>
+    <t>01-trgEntityRelations_SyncClientes.sql</t>
   </si>
   <si>
-    <t>12-AC_pro_ManageGuiasHouseDetallesEditedOrder.sql</t>
+    <t>02-trgUpdateEntityTypes.sql</t>
   </si>
   <si>
-    <t>17-AC_pro_ModuleEdiDetail.sql</t>
+    <t>03-trgUpdateEntities.sql</t>
   </si>
   <si>
-    <t>18-AC_pro_Module_Edi.sql</t>
+    <t>04-f_SearchEntities.sql</t>
   </si>
   <si>
-    <t>28-AC_pro_GetAccountingAnalyticsReports.sql</t>
+    <t>05-AC_pro_General_GenerateBulkInt.sql</t>
   </si>
   <si>
-    <t>24-AC_pro_GetListOFCycleCounts.sql</t>
+    <t>06-AC_pro_GetMachineShipments.sql</t>
   </si>
   <si>
-    <t>29-AC_pro_GetSalesOrders.sql</t>
+    <t>07-AC_pro_GetClientsPiecesDetails.sql</t>
   </si>
   <si>
-    <t>31-AC_pro_GetCompletedScheduledPickupShipTo.sql</t>
+    <t>08-AC_pro_GetDispatchesByCarrier.sql</t>
   </si>
   <si>
-    <t>30-AC_pro_GetDispatchReports.sql</t>
+    <t>09-AC_pro_GetClientsEntities.sql</t>
   </si>
   <si>
-    <t>32-AC_pro_GetCompletedDeliveredPickupShipTo.sql</t>
+    <t>10-AC_pro_GetClientsPiecesBySubCarrier.sql</t>
+  </si>
+  <si>
+    <t>11-AC_pro_GetDispatchesByClient.sql</t>
+  </si>
+  <si>
+    <t>12-AC_pro_GetLocalOrdersByEmployee.sql</t>
+  </si>
+  <si>
+    <t>13-AC_pro_ManageGuiasHouseDetallesEditedOrder.sql</t>
+  </si>
+  <si>
+    <t>14-AC_pro_ListCarrierProgramming.sql</t>
+  </si>
+  <si>
+    <t>15-AC_pro_ConfirmLocalOrderCoordination.sql</t>
+  </si>
+  <si>
+    <t>16-AC_pro_ConfirmLocalOrder.sql</t>
+  </si>
+  <si>
+    <t>17-AC_pro_ShippingDocumentsPODClient360.sql</t>
+  </si>
+  <si>
+    <t>18-AC_pro_ModuleEdiDetail.sql</t>
+  </si>
+  <si>
+    <t>19-AC_pro_Module_Edi.sql</t>
+  </si>
+  <si>
+    <t>20-AC_pro_ListPiecesInventory.sql</t>
+  </si>
+  <si>
+    <t>21-AC_pro_GetBarCodeLinks.sql</t>
+  </si>
+  <si>
+    <t>22-AC_pro_LargeLabelTempDefault.sql</t>
+  </si>
+  <si>
+    <t>23-AC_pro_GetDispatchReports.sql</t>
+  </si>
+  <si>
+    <t>24-AC_pro_GetShipmentAnalyticsReports.sql</t>
+  </si>
+  <si>
+    <t>25-AC_pro_GetListOFCycleCounts.sql</t>
+  </si>
+  <si>
+    <t>26-AC_pro_GetCycleCountDiscrepancies.sql</t>
+  </si>
+  <si>
+    <t>27-AC_pro_CycleCountDiscrepanciesReport.sql</t>
+  </si>
+  <si>
+    <t>28-AC_pro_GetConsolidatedDispatchAnalytics.sql</t>
+  </si>
+  <si>
+    <t>29-AC_pro_GetAccountingAnalyticsReports.sql</t>
+  </si>
+  <si>
+    <t>30-AC_pro_GetSalesOrders.sql</t>
+  </si>
+  <si>
+    <t>31-AC_pro_GetDispatchReports.sql</t>
+  </si>
+  <si>
+    <t>32-AC_pro_GetCompletedScheduledPickupShipTo.sql</t>
+  </si>
+  <si>
+    <t>33-AC_pro_GetCompletedDeliveredPickupShipTo.sql</t>
   </si>
 </sst>
 </file>
@@ -826,7 +829,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="78">
+  <borders count="79">
     <border>
       <left/>
       <right/>
@@ -1811,12 +1814,23 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="173">
+  <cellXfs count="176">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1969,8 +1983,83 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="75" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="76" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="77" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="52" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="60" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="61" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="65" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="62" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="66" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="40" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="55" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="71" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="51" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="52" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="53" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="72" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="73" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="74" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2074,84 +2163,6 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="60" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="61" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="65" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="62" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="66" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="40" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="55" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="71" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="51" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="52" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="53" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="72" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="73" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="74" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="52" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="10" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2224,6 +2235,9 @@
     <xf numFmtId="0" fontId="0" fillId="11" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="9" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2247,6 +2261,15 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="78" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="51" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="54" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2311,7 +2334,7 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp109.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="Hoja4!$A$1:$A$25" noThreeD="1" sel="17" val="14"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="Hoja4!$A$1:$A$25" noThreeD="1" sel="23" val="16"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp11.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2319,7 +2342,7 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp110.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="Hoja4!$A$1:$A$25" noThreeD="1" sel="8" val="7"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="Hoja4!$A$1:$A$25" noThreeD="1" sel="17" val="12"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp111.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2439,7 +2462,7 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp138.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="Hoja4!$A$1:$A$17" noThreeD="1" sel="17" val="9"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="Hoja4!$A$1:$A$18" noThreeD="1" sel="8" val="3"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp139.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2448,6 +2471,10 @@
 
 <file path=xl/ctrlProps/ctrlProp14.xml><?xml version="1.0" encoding="utf-8"?>
 <formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="[1]Hoja4!$A$1:$A$13" noThreeD="1" sel="0" val="0"/>
+</file>
+
+<file path=xl/ctrlProps/ctrlProp140.xml><?xml version="1.0" encoding="utf-8"?>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Drop" dropStyle="combo" dx="26" fmlaRange="Hoja4!$A$1:$A$17" noThreeD="1" sel="17" val="9"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp15.xml><?xml version="1.0" encoding="utf-8"?>
@@ -10609,7 +10636,7 @@
           <xdr:col>2</xdr:col>
           <xdr:colOff>1409700</xdr:colOff>
           <xdr:row>55</xdr:row>
-          <xdr:rowOff>2241</xdr:rowOff>
+          <xdr:rowOff>7620</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -10667,7 +10694,7 @@
           <xdr:col>2</xdr:col>
           <xdr:colOff>1409700</xdr:colOff>
           <xdr:row>56</xdr:row>
-          <xdr:rowOff>2241</xdr:rowOff>
+          <xdr:rowOff>7620</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -10725,7 +10752,7 @@
           <xdr:col>2</xdr:col>
           <xdr:colOff>1409700</xdr:colOff>
           <xdr:row>57</xdr:row>
-          <xdr:rowOff>2241</xdr:rowOff>
+          <xdr:rowOff>7620</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -10735,7 +10762,65 @@
                   <a14:compatExt spid="_x0000_s1239"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B5306AB2-C689-6E6B-B36B-1B34C0356C8E}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-0000D7040000}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="0" cy="0"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:extLst>
+              <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
+                <a14:hiddenLine w="9525">
+                  <a:noFill/>
+                  <a:miter lim="800000"/>
+                  <a:headEnd/>
+                  <a:tailEnd/>
+                </a14:hiddenLine>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+        </xdr:sp>
+        <xdr:clientData/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:twoCellAnchor editAs="oneCell">
+        <xdr:from>
+          <xdr:col>2</xdr:col>
+          <xdr:colOff>0</xdr:colOff>
+          <xdr:row>57</xdr:row>
+          <xdr:rowOff>0</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>2</xdr:col>
+          <xdr:colOff>1409700</xdr:colOff>
+          <xdr:row>58</xdr:row>
+          <xdr:rowOff>38100</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="1240" name="Drop Down 216" hidden="1">
+              <a:extLst>
+                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
+                  <a14:compatExt spid="_x0000_s1240"/>
+                </a:ext>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FF2454DC-C779-3BA6-DA50-36A79288A231}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -11361,7 +11446,7 @@
   <sheetPr codeName="Hoja1">
     <tabColor theme="9"/>
   </sheetPr>
-  <dimension ref="A3:O57"/>
+  <dimension ref="A3:O58"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="35.44140625" bestFit="1" customWidth="1"/>
@@ -11380,42 +11465,42 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:15" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="97" t="s">
+      <c r="A3" s="122" t="s">
         <v>103</v>
       </c>
-      <c r="B3" s="98"/>
-      <c r="C3" s="98"/>
-      <c r="D3" s="98"/>
-      <c r="E3" s="98"/>
-      <c r="F3" s="98"/>
-      <c r="G3" s="98"/>
-      <c r="H3" s="98"/>
-      <c r="I3" s="98"/>
-      <c r="J3" s="98"/>
-      <c r="K3" s="98"/>
-      <c r="L3" s="99"/>
-      <c r="N3" s="91" t="s">
+      <c r="B3" s="123"/>
+      <c r="C3" s="123"/>
+      <c r="D3" s="123"/>
+      <c r="E3" s="123"/>
+      <c r="F3" s="123"/>
+      <c r="G3" s="123"/>
+      <c r="H3" s="123"/>
+      <c r="I3" s="123"/>
+      <c r="J3" s="123"/>
+      <c r="K3" s="123"/>
+      <c r="L3" s="124"/>
+      <c r="N3" s="116" t="s">
         <v>0</v>
       </c>
-      <c r="O3" s="92"/>
+      <c r="O3" s="117"/>
     </row>
     <row r="4" spans="1:15" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="104" t="s">
+      <c r="B4" s="129" t="s">
         <v>105</v>
       </c>
-      <c r="C4" s="105"/>
-      <c r="D4" s="105"/>
-      <c r="E4" s="105"/>
-      <c r="F4" s="105"/>
-      <c r="G4" s="105"/>
-      <c r="H4" s="105"/>
-      <c r="I4" s="105"/>
-      <c r="J4" s="106"/>
-      <c r="K4" s="106"/>
-      <c r="L4" s="107"/>
+      <c r="C4" s="130"/>
+      <c r="D4" s="130"/>
+      <c r="E4" s="130"/>
+      <c r="F4" s="130"/>
+      <c r="G4" s="130"/>
+      <c r="H4" s="130"/>
+      <c r="I4" s="130"/>
+      <c r="J4" s="131"/>
+      <c r="K4" s="131"/>
+      <c r="L4" s="132"/>
       <c r="N4" s="21" t="s">
         <v>2</v>
       </c>
@@ -11425,19 +11510,19 @@
       <c r="A5" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="108" t="s">
+      <c r="B5" s="133" t="s">
         <v>109</v>
       </c>
-      <c r="C5" s="108"/>
-      <c r="D5" s="108"/>
-      <c r="E5" s="108"/>
-      <c r="F5" s="108"/>
-      <c r="G5" s="108"/>
-      <c r="H5" s="108"/>
-      <c r="I5" s="108"/>
-      <c r="J5" s="109"/>
-      <c r="K5" s="109"/>
-      <c r="L5" s="110"/>
+      <c r="C5" s="133"/>
+      <c r="D5" s="133"/>
+      <c r="E5" s="133"/>
+      <c r="F5" s="133"/>
+      <c r="G5" s="133"/>
+      <c r="H5" s="133"/>
+      <c r="I5" s="133"/>
+      <c r="J5" s="134"/>
+      <c r="K5" s="134"/>
+      <c r="L5" s="135"/>
       <c r="N5" s="15" t="s">
         <v>4</v>
       </c>
@@ -11447,19 +11532,19 @@
       <c r="A6" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="94">
+      <c r="B6" s="119">
         <v>46073</v>
       </c>
-      <c r="C6" s="95"/>
-      <c r="D6" s="95"/>
-      <c r="E6" s="95"/>
-      <c r="F6" s="95"/>
-      <c r="G6" s="95"/>
-      <c r="H6" s="95"/>
-      <c r="I6" s="95"/>
-      <c r="J6" s="95"/>
-      <c r="K6" s="95"/>
-      <c r="L6" s="96"/>
+      <c r="C6" s="120"/>
+      <c r="D6" s="120"/>
+      <c r="E6" s="120"/>
+      <c r="F6" s="120"/>
+      <c r="G6" s="120"/>
+      <c r="H6" s="120"/>
+      <c r="I6" s="120"/>
+      <c r="J6" s="120"/>
+      <c r="K6" s="120"/>
+      <c r="L6" s="121"/>
       <c r="N6" s="14"/>
       <c r="O6" s="14"/>
     </row>
@@ -11467,17 +11552,17 @@
       <c r="A7" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="111"/>
-      <c r="C7" s="112"/>
-      <c r="D7" s="112"/>
-      <c r="E7" s="112"/>
-      <c r="F7" s="112"/>
-      <c r="G7" s="112"/>
-      <c r="H7" s="112"/>
-      <c r="I7" s="112"/>
-      <c r="J7" s="113"/>
-      <c r="K7" s="113"/>
-      <c r="L7" s="114"/>
+      <c r="B7" s="136"/>
+      <c r="C7" s="137"/>
+      <c r="D7" s="137"/>
+      <c r="E7" s="137"/>
+      <c r="F7" s="137"/>
+      <c r="G7" s="137"/>
+      <c r="H7" s="137"/>
+      <c r="I7" s="137"/>
+      <c r="J7" s="138"/>
+      <c r="K7" s="138"/>
+      <c r="L7" s="139"/>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" s="11"/>
@@ -11494,20 +11579,20 @@
       <c r="L8" s="13"/>
     </row>
     <row r="9" spans="1:15" s="5" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="100" t="s">
+      <c r="A9" s="125" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="101"/>
-      <c r="C9" s="101"/>
-      <c r="D9" s="101"/>
-      <c r="E9" s="101"/>
-      <c r="F9" s="101"/>
-      <c r="G9" s="101"/>
-      <c r="H9" s="101"/>
-      <c r="I9" s="101"/>
-      <c r="J9" s="102"/>
-      <c r="K9" s="102"/>
-      <c r="L9" s="103"/>
+      <c r="B9" s="126"/>
+      <c r="C9" s="126"/>
+      <c r="D9" s="126"/>
+      <c r="E9" s="126"/>
+      <c r="F9" s="126"/>
+      <c r="G9" s="126"/>
+      <c r="H9" s="126"/>
+      <c r="I9" s="126"/>
+      <c r="J9" s="127"/>
+      <c r="K9" s="127"/>
+      <c r="L9" s="128"/>
     </row>
     <row r="10" spans="1:15" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
@@ -11607,63 +11692,63 @@
       <c r="A14" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="B14" s="93"/>
-      <c r="C14" s="89"/>
-      <c r="D14" s="89"/>
-      <c r="E14" s="89"/>
-      <c r="F14" s="89"/>
-      <c r="G14" s="89"/>
-      <c r="H14" s="89"/>
-      <c r="I14" s="89"/>
-      <c r="J14" s="89"/>
-      <c r="K14" s="89"/>
-      <c r="L14" s="90"/>
+      <c r="B14" s="118"/>
+      <c r="C14" s="114"/>
+      <c r="D14" s="114"/>
+      <c r="E14" s="114"/>
+      <c r="F14" s="114"/>
+      <c r="G14" s="114"/>
+      <c r="H14" s="114"/>
+      <c r="I14" s="114"/>
+      <c r="J14" s="114"/>
+      <c r="K14" s="114"/>
+      <c r="L14" s="115"/>
     </row>
     <row r="15" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="B15" s="88"/>
-      <c r="C15" s="89"/>
-      <c r="D15" s="89"/>
-      <c r="E15" s="89"/>
-      <c r="F15" s="89"/>
-      <c r="G15" s="89"/>
-      <c r="H15" s="89"/>
-      <c r="I15" s="89"/>
-      <c r="J15" s="89"/>
-      <c r="K15" s="89"/>
-      <c r="L15" s="90"/>
+      <c r="B15" s="113"/>
+      <c r="C15" s="114"/>
+      <c r="D15" s="114"/>
+      <c r="E15" s="114"/>
+      <c r="F15" s="114"/>
+      <c r="G15" s="114"/>
+      <c r="H15" s="114"/>
+      <c r="I15" s="114"/>
+      <c r="J15" s="114"/>
+      <c r="K15" s="114"/>
+      <c r="L15" s="115"/>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A16" s="81"/>
-      <c r="B16" s="82"/>
-      <c r="C16" s="82"/>
-      <c r="D16" s="82"/>
-      <c r="E16" s="82"/>
-      <c r="F16" s="82"/>
-      <c r="G16" s="82"/>
-      <c r="H16" s="82"/>
-      <c r="I16" s="82"/>
-      <c r="J16" s="82"/>
-      <c r="K16" s="82"/>
-      <c r="L16" s="83"/>
+      <c r="A16" s="106"/>
+      <c r="B16" s="107"/>
+      <c r="C16" s="107"/>
+      <c r="D16" s="107"/>
+      <c r="E16" s="107"/>
+      <c r="F16" s="107"/>
+      <c r="G16" s="107"/>
+      <c r="H16" s="107"/>
+      <c r="I16" s="107"/>
+      <c r="J16" s="107"/>
+      <c r="K16" s="107"/>
+      <c r="L16" s="108"/>
     </row>
     <row r="17" spans="1:12" s="5" customFormat="1" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="84" t="s">
+      <c r="A17" s="109" t="s">
         <v>25</v>
       </c>
-      <c r="B17" s="85"/>
-      <c r="C17" s="85"/>
-      <c r="D17" s="85"/>
-      <c r="E17" s="85"/>
-      <c r="F17" s="85"/>
-      <c r="G17" s="85"/>
-      <c r="H17" s="85"/>
-      <c r="I17" s="85"/>
-      <c r="J17" s="86"/>
-      <c r="K17" s="86"/>
-      <c r="L17" s="87"/>
+      <c r="B17" s="110"/>
+      <c r="C17" s="110"/>
+      <c r="D17" s="110"/>
+      <c r="E17" s="110"/>
+      <c r="F17" s="110"/>
+      <c r="G17" s="110"/>
+      <c r="H17" s="110"/>
+      <c r="I17" s="110"/>
+      <c r="J17" s="111"/>
+      <c r="K17" s="111"/>
+      <c r="L17" s="112"/>
     </row>
     <row r="18" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="6"/>
@@ -11673,19 +11758,19 @@
       <c r="C18" s="43" t="s">
         <v>27</v>
       </c>
-      <c r="D18" s="115" t="s">
+      <c r="D18" s="82" t="s">
         <v>28</v>
       </c>
-      <c r="E18" s="117" t="s">
-        <v>137</v>
-      </c>
-      <c r="F18" s="117"/>
-      <c r="G18" s="117"/>
-      <c r="H18" s="117"/>
-      <c r="I18" s="117"/>
-      <c r="J18" s="118"/>
-      <c r="K18" s="118"/>
-      <c r="L18" s="119"/>
+      <c r="E18" s="84" t="s">
+        <v>115</v>
+      </c>
+      <c r="F18" s="84"/>
+      <c r="G18" s="84"/>
+      <c r="H18" s="84"/>
+      <c r="I18" s="84"/>
+      <c r="J18" s="85"/>
+      <c r="K18" s="85"/>
+      <c r="L18" s="86"/>
     </row>
     <row r="19" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="8" t="s">
@@ -11695,15 +11780,15 @@
         <v>30</v>
       </c>
       <c r="C19" s="44"/>
-      <c r="D19" s="116"/>
-      <c r="E19" s="120"/>
-      <c r="F19" s="120"/>
-      <c r="G19" s="120"/>
-      <c r="H19" s="120"/>
-      <c r="I19" s="120"/>
-      <c r="J19" s="121"/>
-      <c r="K19" s="121"/>
-      <c r="L19" s="122"/>
+      <c r="D19" s="83"/>
+      <c r="E19" s="87"/>
+      <c r="F19" s="87"/>
+      <c r="G19" s="87"/>
+      <c r="H19" s="87"/>
+      <c r="I19" s="87"/>
+      <c r="J19" s="88"/>
+      <c r="K19" s="88"/>
+      <c r="L19" s="89"/>
     </row>
     <row r="20" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="8" t="s">
@@ -11713,15 +11798,15 @@
       <c r="C20" s="44" t="s">
         <v>30</v>
       </c>
-      <c r="D20" s="116"/>
-      <c r="E20" s="120"/>
-      <c r="F20" s="120"/>
-      <c r="G20" s="120"/>
-      <c r="H20" s="120"/>
-      <c r="I20" s="120"/>
-      <c r="J20" s="121"/>
-      <c r="K20" s="121"/>
-      <c r="L20" s="122"/>
+      <c r="D20" s="83"/>
+      <c r="E20" s="87"/>
+      <c r="F20" s="87"/>
+      <c r="G20" s="87"/>
+      <c r="H20" s="87"/>
+      <c r="I20" s="87"/>
+      <c r="J20" s="88"/>
+      <c r="K20" s="88"/>
+      <c r="L20" s="89"/>
     </row>
     <row r="21" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="8" t="s">
@@ -11731,19 +11816,19 @@
       <c r="C21" s="44" t="s">
         <v>30</v>
       </c>
-      <c r="D21" s="131" t="s">
+      <c r="D21" s="98" t="s">
         <v>25</v>
       </c>
-      <c r="E21" s="133" t="s">
+      <c r="E21" s="100" t="s">
         <v>107</v>
       </c>
-      <c r="F21" s="134"/>
-      <c r="G21" s="134"/>
-      <c r="H21" s="134"/>
-      <c r="I21" s="134"/>
-      <c r="J21" s="134"/>
-      <c r="K21" s="134"/>
-      <c r="L21" s="135"/>
+      <c r="F21" s="101"/>
+      <c r="G21" s="101"/>
+      <c r="H21" s="101"/>
+      <c r="I21" s="101"/>
+      <c r="J21" s="101"/>
+      <c r="K21" s="101"/>
+      <c r="L21" s="102"/>
     </row>
     <row r="22" spans="1:12" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="8" t="s">
@@ -11753,45 +11838,45 @@
       <c r="C22" s="44" t="s">
         <v>30</v>
       </c>
-      <c r="D22" s="132"/>
-      <c r="E22" s="136"/>
-      <c r="F22" s="137"/>
-      <c r="G22" s="137"/>
-      <c r="H22" s="137"/>
-      <c r="I22" s="137"/>
-      <c r="J22" s="137"/>
-      <c r="K22" s="137"/>
-      <c r="L22" s="138"/>
+      <c r="D22" s="99"/>
+      <c r="E22" s="103"/>
+      <c r="F22" s="104"/>
+      <c r="G22" s="104"/>
+      <c r="H22" s="104"/>
+      <c r="I22" s="104"/>
+      <c r="J22" s="104"/>
+      <c r="K22" s="104"/>
+      <c r="L22" s="105"/>
     </row>
     <row r="23" spans="1:12" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="124"/>
-      <c r="B23" s="125"/>
-      <c r="C23" s="125"/>
-      <c r="D23" s="126"/>
-      <c r="E23" s="126"/>
-      <c r="F23" s="126"/>
-      <c r="G23" s="126"/>
-      <c r="H23" s="126"/>
-      <c r="I23" s="126"/>
-      <c r="J23" s="126"/>
-      <c r="K23" s="126"/>
-      <c r="L23" s="127"/>
+      <c r="A23" s="91"/>
+      <c r="B23" s="92"/>
+      <c r="C23" s="92"/>
+      <c r="D23" s="93"/>
+      <c r="E23" s="93"/>
+      <c r="F23" s="93"/>
+      <c r="G23" s="93"/>
+      <c r="H23" s="93"/>
+      <c r="I23" s="93"/>
+      <c r="J23" s="93"/>
+      <c r="K23" s="93"/>
+      <c r="L23" s="94"/>
     </row>
     <row r="24" spans="1:12" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A24" s="128" t="s">
+      <c r="A24" s="95" t="s">
         <v>34</v>
       </c>
-      <c r="B24" s="129"/>
-      <c r="C24" s="129"/>
-      <c r="D24" s="129"/>
-      <c r="E24" s="129"/>
-      <c r="F24" s="129"/>
-      <c r="G24" s="129"/>
-      <c r="H24" s="129"/>
-      <c r="I24" s="129"/>
-      <c r="J24" s="129"/>
-      <c r="K24" s="129"/>
-      <c r="L24" s="130"/>
+      <c r="B24" s="96"/>
+      <c r="C24" s="96"/>
+      <c r="D24" s="96"/>
+      <c r="E24" s="96"/>
+      <c r="F24" s="96"/>
+      <c r="G24" s="96"/>
+      <c r="H24" s="96"/>
+      <c r="I24" s="96"/>
+      <c r="J24" s="96"/>
+      <c r="K24" s="96"/>
+      <c r="L24" s="97"/>
     </row>
     <row r="25" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A25" s="16" t="s">
@@ -11803,523 +11888,523 @@
       <c r="C25" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="D25" s="123" t="s">
+      <c r="D25" s="90" t="s">
         <v>38</v>
       </c>
-      <c r="E25" s="123"/>
-      <c r="F25" s="123"/>
-      <c r="G25" s="123"/>
-      <c r="H25" s="123"/>
-      <c r="I25" s="123"/>
-      <c r="J25" s="123"/>
-      <c r="K25" s="123"/>
-      <c r="L25" s="123"/>
+      <c r="E25" s="90"/>
+      <c r="F25" s="90"/>
+      <c r="G25" s="90"/>
+      <c r="H25" s="90"/>
+      <c r="I25" s="90"/>
+      <c r="J25" s="90"/>
+      <c r="K25" s="90"/>
+      <c r="L25" s="90"/>
     </row>
     <row r="26" spans="1:12" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="33">
         <v>1</v>
       </c>
       <c r="B26" s="34" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C26" s="34"/>
-      <c r="D26" s="139" t="s">
+      <c r="D26" s="174" t="s">
         <v>108</v>
       </c>
-      <c r="E26" s="139"/>
-      <c r="F26" s="139"/>
-      <c r="G26" s="139"/>
-      <c r="H26" s="139"/>
-      <c r="I26" s="139"/>
-      <c r="J26" s="139"/>
-      <c r="K26" s="139"/>
-      <c r="L26" s="139"/>
+      <c r="E26" s="80"/>
+      <c r="F26" s="80"/>
+      <c r="G26" s="80"/>
+      <c r="H26" s="80"/>
+      <c r="I26" s="80"/>
+      <c r="J26" s="80"/>
+      <c r="K26" s="80"/>
+      <c r="L26" s="80"/>
     </row>
     <row r="27" spans="1:12" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="33">
         <v>2</v>
       </c>
       <c r="B27" s="34" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C27" s="34"/>
-      <c r="D27" s="140"/>
-      <c r="E27" s="140"/>
-      <c r="F27" s="140"/>
-      <c r="G27" s="140"/>
-      <c r="H27" s="140"/>
-      <c r="I27" s="140"/>
-      <c r="J27" s="140"/>
-      <c r="K27" s="140"/>
-      <c r="L27" s="140"/>
+      <c r="D27" s="175"/>
+      <c r="E27" s="81"/>
+      <c r="F27" s="81"/>
+      <c r="G27" s="81"/>
+      <c r="H27" s="81"/>
+      <c r="I27" s="81"/>
+      <c r="J27" s="81"/>
+      <c r="K27" s="81"/>
+      <c r="L27" s="81"/>
     </row>
     <row r="28" spans="1:12" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="33">
         <v>3</v>
       </c>
       <c r="B28" s="34" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C28" s="34"/>
-      <c r="D28" s="140"/>
-      <c r="E28" s="140"/>
-      <c r="F28" s="140"/>
-      <c r="G28" s="140"/>
-      <c r="H28" s="140"/>
-      <c r="I28" s="140"/>
-      <c r="J28" s="140"/>
-      <c r="K28" s="140"/>
-      <c r="L28" s="140"/>
+      <c r="D28" s="175"/>
+      <c r="E28" s="81"/>
+      <c r="F28" s="81"/>
+      <c r="G28" s="81"/>
+      <c r="H28" s="81"/>
+      <c r="I28" s="81"/>
+      <c r="J28" s="81"/>
+      <c r="K28" s="81"/>
+      <c r="L28" s="81"/>
     </row>
     <row r="29" spans="1:12" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="33">
         <v>4</v>
       </c>
       <c r="B29" s="34" t="s">
-        <v>138</v>
+        <v>119</v>
       </c>
       <c r="C29" s="34"/>
-      <c r="D29" s="140"/>
-      <c r="E29" s="140"/>
-      <c r="F29" s="140"/>
-      <c r="G29" s="140"/>
-      <c r="H29" s="140"/>
-      <c r="I29" s="140"/>
-      <c r="J29" s="140"/>
-      <c r="K29" s="140"/>
-      <c r="L29" s="140"/>
+      <c r="D29" s="175"/>
+      <c r="E29" s="81"/>
+      <c r="F29" s="81"/>
+      <c r="G29" s="81"/>
+      <c r="H29" s="81"/>
+      <c r="I29" s="81"/>
+      <c r="J29" s="81"/>
+      <c r="K29" s="81"/>
+      <c r="L29" s="81"/>
     </row>
     <row r="30" spans="1:12" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="33">
         <v>5</v>
       </c>
       <c r="B30" s="34" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C30" s="34"/>
-      <c r="D30" s="140"/>
-      <c r="E30" s="140"/>
-      <c r="F30" s="140"/>
-      <c r="G30" s="140"/>
-      <c r="H30" s="140"/>
-      <c r="I30" s="140"/>
-      <c r="J30" s="140"/>
-      <c r="K30" s="140"/>
-      <c r="L30" s="140"/>
+      <c r="D30" s="175"/>
+      <c r="E30" s="81"/>
+      <c r="F30" s="81"/>
+      <c r="G30" s="81"/>
+      <c r="H30" s="81"/>
+      <c r="I30" s="81"/>
+      <c r="J30" s="81"/>
+      <c r="K30" s="81"/>
+      <c r="L30" s="81"/>
     </row>
     <row r="31" spans="1:12" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="33">
         <v>6</v>
       </c>
       <c r="B31" s="34" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C31" s="34"/>
-      <c r="D31" s="140"/>
-      <c r="E31" s="140"/>
-      <c r="F31" s="140"/>
-      <c r="G31" s="140"/>
-      <c r="H31" s="140"/>
-      <c r="I31" s="140"/>
-      <c r="J31" s="140"/>
-      <c r="K31" s="140"/>
-      <c r="L31" s="140"/>
+      <c r="D31" s="175"/>
+      <c r="E31" s="81"/>
+      <c r="F31" s="81"/>
+      <c r="G31" s="81"/>
+      <c r="H31" s="81"/>
+      <c r="I31" s="81"/>
+      <c r="J31" s="81"/>
+      <c r="K31" s="81"/>
+      <c r="L31" s="81"/>
     </row>
     <row r="32" spans="1:12" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="33">
         <v>7</v>
       </c>
       <c r="B32" s="34" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C32" s="34"/>
-      <c r="D32" s="140"/>
-      <c r="E32" s="140"/>
-      <c r="F32" s="140"/>
-      <c r="G32" s="140"/>
-      <c r="H32" s="140"/>
-      <c r="I32" s="140"/>
-      <c r="J32" s="140"/>
-      <c r="K32" s="140"/>
-      <c r="L32" s="140"/>
+      <c r="D32" s="175"/>
+      <c r="E32" s="81"/>
+      <c r="F32" s="81"/>
+      <c r="G32" s="81"/>
+      <c r="H32" s="81"/>
+      <c r="I32" s="81"/>
+      <c r="J32" s="81"/>
+      <c r="K32" s="81"/>
+      <c r="L32" s="81"/>
     </row>
     <row r="33" spans="1:12" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="33">
         <v>8</v>
       </c>
       <c r="B33" s="34" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C33" s="34"/>
-      <c r="D33" s="140"/>
-      <c r="E33" s="140"/>
-      <c r="F33" s="140"/>
-      <c r="G33" s="140"/>
-      <c r="H33" s="140"/>
-      <c r="I33" s="140"/>
-      <c r="J33" s="140"/>
-      <c r="K33" s="140"/>
-      <c r="L33" s="140"/>
+      <c r="D33" s="175"/>
+      <c r="E33" s="81"/>
+      <c r="F33" s="81"/>
+      <c r="G33" s="81"/>
+      <c r="H33" s="81"/>
+      <c r="I33" s="81"/>
+      <c r="J33" s="81"/>
+      <c r="K33" s="81"/>
+      <c r="L33" s="81"/>
     </row>
     <row r="34" spans="1:12" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="33">
         <v>9</v>
       </c>
       <c r="B34" s="34" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C34" s="34"/>
-      <c r="D34" s="140"/>
-      <c r="E34" s="140"/>
-      <c r="F34" s="140"/>
-      <c r="G34" s="140"/>
-      <c r="H34" s="140"/>
-      <c r="I34" s="140"/>
-      <c r="J34" s="140"/>
-      <c r="K34" s="140"/>
-      <c r="L34" s="140"/>
+      <c r="D34" s="175"/>
+      <c r="E34" s="81"/>
+      <c r="F34" s="81"/>
+      <c r="G34" s="81"/>
+      <c r="H34" s="81"/>
+      <c r="I34" s="81"/>
+      <c r="J34" s="81"/>
+      <c r="K34" s="81"/>
+      <c r="L34" s="81"/>
     </row>
     <row r="35" spans="1:12" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="33">
         <v>10</v>
       </c>
       <c r="B35" s="34" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C35" s="34"/>
-      <c r="D35" s="140"/>
-      <c r="E35" s="140"/>
-      <c r="F35" s="140"/>
-      <c r="G35" s="140"/>
-      <c r="H35" s="140"/>
-      <c r="I35" s="140"/>
-      <c r="J35" s="140"/>
-      <c r="K35" s="140"/>
-      <c r="L35" s="140"/>
+      <c r="D35" s="175"/>
+      <c r="E35" s="81"/>
+      <c r="F35" s="81"/>
+      <c r="G35" s="81"/>
+      <c r="H35" s="81"/>
+      <c r="I35" s="81"/>
+      <c r="J35" s="81"/>
+      <c r="K35" s="81"/>
+      <c r="L35" s="81"/>
     </row>
     <row r="36" spans="1:12" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="33">
         <v>11</v>
       </c>
       <c r="B36" s="34" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C36" s="34"/>
-      <c r="D36" s="140"/>
-      <c r="E36" s="140"/>
-      <c r="F36" s="140"/>
-      <c r="G36" s="140"/>
-      <c r="H36" s="140"/>
-      <c r="I36" s="140"/>
-      <c r="J36" s="140"/>
-      <c r="K36" s="140"/>
-      <c r="L36" s="140"/>
+      <c r="D36" s="175"/>
+      <c r="E36" s="81"/>
+      <c r="F36" s="81"/>
+      <c r="G36" s="81"/>
+      <c r="H36" s="81"/>
+      <c r="I36" s="81"/>
+      <c r="J36" s="81"/>
+      <c r="K36" s="81"/>
+      <c r="L36" s="81"/>
     </row>
     <row r="37" spans="1:12" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="33">
         <v>12</v>
       </c>
       <c r="B37" s="34" t="s">
-        <v>139</v>
+        <v>127</v>
       </c>
       <c r="C37" s="34"/>
-      <c r="D37" s="140"/>
-      <c r="E37" s="140"/>
-      <c r="F37" s="140"/>
-      <c r="G37" s="140"/>
-      <c r="H37" s="140"/>
-      <c r="I37" s="140"/>
-      <c r="J37" s="140"/>
-      <c r="K37" s="140"/>
-      <c r="L37" s="140"/>
+      <c r="D37" s="175"/>
+      <c r="E37" s="81"/>
+      <c r="F37" s="81"/>
+      <c r="G37" s="81"/>
+      <c r="H37" s="81"/>
+      <c r="I37" s="81"/>
+      <c r="J37" s="81"/>
+      <c r="K37" s="81"/>
+      <c r="L37" s="81"/>
     </row>
     <row r="38" spans="1:12" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="33">
         <v>13</v>
       </c>
       <c r="B38" s="34" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="C38" s="34"/>
-      <c r="D38" s="140"/>
-      <c r="E38" s="140"/>
-      <c r="F38" s="140"/>
-      <c r="G38" s="140"/>
-      <c r="H38" s="140"/>
-      <c r="I38" s="140"/>
-      <c r="J38" s="140"/>
-      <c r="K38" s="140"/>
-      <c r="L38" s="140"/>
+      <c r="D38" s="175"/>
+      <c r="E38" s="81"/>
+      <c r="F38" s="81"/>
+      <c r="G38" s="81"/>
+      <c r="H38" s="81"/>
+      <c r="I38" s="81"/>
+      <c r="J38" s="81"/>
+      <c r="K38" s="81"/>
+      <c r="L38" s="81"/>
     </row>
     <row r="39" spans="1:12" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="33">
         <v>14</v>
       </c>
       <c r="B39" s="34" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="C39" s="34"/>
-      <c r="D39" s="140"/>
-      <c r="E39" s="140"/>
-      <c r="F39" s="140"/>
-      <c r="G39" s="140"/>
-      <c r="H39" s="140"/>
-      <c r="I39" s="140"/>
-      <c r="J39" s="140"/>
-      <c r="K39" s="140"/>
-      <c r="L39" s="140"/>
+      <c r="D39" s="175"/>
+      <c r="E39" s="81"/>
+      <c r="F39" s="81"/>
+      <c r="G39" s="81"/>
+      <c r="H39" s="81"/>
+      <c r="I39" s="81"/>
+      <c r="J39" s="81"/>
+      <c r="K39" s="81"/>
+      <c r="L39" s="81"/>
     </row>
     <row r="40" spans="1:12" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="33">
         <v>15</v>
       </c>
       <c r="B40" s="34" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="C40" s="34"/>
-      <c r="D40" s="140"/>
-      <c r="E40" s="140"/>
-      <c r="F40" s="140"/>
-      <c r="G40" s="140"/>
-      <c r="H40" s="140"/>
-      <c r="I40" s="140"/>
-      <c r="J40" s="140"/>
-      <c r="K40" s="140"/>
-      <c r="L40" s="140"/>
+      <c r="D40" s="175"/>
+      <c r="E40" s="81"/>
+      <c r="F40" s="81"/>
+      <c r="G40" s="81"/>
+      <c r="H40" s="81"/>
+      <c r="I40" s="81"/>
+      <c r="J40" s="81"/>
+      <c r="K40" s="81"/>
+      <c r="L40" s="81"/>
     </row>
     <row r="41" spans="1:12" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="33">
         <v>16</v>
       </c>
       <c r="B41" s="34" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="C41" s="34"/>
-      <c r="D41" s="140"/>
-      <c r="E41" s="140"/>
-      <c r="F41" s="140"/>
-      <c r="G41" s="140"/>
-      <c r="H41" s="140"/>
-      <c r="I41" s="140"/>
-      <c r="J41" s="140"/>
-      <c r="K41" s="140"/>
-      <c r="L41" s="140"/>
+      <c r="D41" s="175"/>
+      <c r="E41" s="81"/>
+      <c r="F41" s="81"/>
+      <c r="G41" s="81"/>
+      <c r="H41" s="81"/>
+      <c r="I41" s="81"/>
+      <c r="J41" s="81"/>
+      <c r="K41" s="81"/>
+      <c r="L41" s="81"/>
     </row>
     <row r="42" spans="1:12" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="33">
         <v>17</v>
       </c>
       <c r="B42" s="34" t="s">
-        <v>140</v>
+        <v>132</v>
       </c>
       <c r="C42" s="34"/>
-      <c r="D42" s="140"/>
-      <c r="E42" s="140"/>
-      <c r="F42" s="140"/>
-      <c r="G42" s="140"/>
-      <c r="H42" s="140"/>
-      <c r="I42" s="140"/>
-      <c r="J42" s="140"/>
-      <c r="K42" s="140"/>
-      <c r="L42" s="140"/>
+      <c r="D42" s="175"/>
+      <c r="E42" s="81"/>
+      <c r="F42" s="81"/>
+      <c r="G42" s="81"/>
+      <c r="H42" s="81"/>
+      <c r="I42" s="81"/>
+      <c r="J42" s="81"/>
+      <c r="K42" s="81"/>
+      <c r="L42" s="81"/>
     </row>
     <row r="43" spans="1:12" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="33">
         <v>18</v>
       </c>
       <c r="B43" s="34" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="C43" s="34"/>
-      <c r="D43" s="140"/>
-      <c r="E43" s="140"/>
-      <c r="F43" s="140"/>
-      <c r="G43" s="140"/>
-      <c r="H43" s="140"/>
-      <c r="I43" s="140"/>
-      <c r="J43" s="140"/>
-      <c r="K43" s="140"/>
-      <c r="L43" s="140"/>
+      <c r="D43" s="175"/>
+      <c r="E43" s="81"/>
+      <c r="F43" s="81"/>
+      <c r="G43" s="81"/>
+      <c r="H43" s="81"/>
+      <c r="I43" s="81"/>
+      <c r="J43" s="81"/>
+      <c r="K43" s="81"/>
+      <c r="L43" s="81"/>
     </row>
     <row r="44" spans="1:12" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="33">
         <v>19</v>
       </c>
       <c r="B44" s="34" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="C44" s="34"/>
-      <c r="D44" s="140"/>
-      <c r="E44" s="140"/>
-      <c r="F44" s="140"/>
-      <c r="G44" s="140"/>
-      <c r="H44" s="140"/>
-      <c r="I44" s="140"/>
-      <c r="J44" s="140"/>
-      <c r="K44" s="140"/>
-      <c r="L44" s="140"/>
+      <c r="D44" s="175"/>
+      <c r="E44" s="81"/>
+      <c r="F44" s="81"/>
+      <c r="G44" s="81"/>
+      <c r="H44" s="81"/>
+      <c r="I44" s="81"/>
+      <c r="J44" s="81"/>
+      <c r="K44" s="81"/>
+      <c r="L44" s="81"/>
     </row>
     <row r="45" spans="1:12" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="33">
         <v>20</v>
       </c>
       <c r="B45" s="34" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="C45" s="34"/>
-      <c r="D45" s="140"/>
-      <c r="E45" s="140"/>
-      <c r="F45" s="140"/>
-      <c r="G45" s="140"/>
-      <c r="H45" s="140"/>
-      <c r="I45" s="140"/>
-      <c r="J45" s="140"/>
-      <c r="K45" s="140"/>
-      <c r="L45" s="140"/>
+      <c r="D45" s="175"/>
+      <c r="E45" s="81"/>
+      <c r="F45" s="81"/>
+      <c r="G45" s="81"/>
+      <c r="H45" s="81"/>
+      <c r="I45" s="81"/>
+      <c r="J45" s="81"/>
+      <c r="K45" s="81"/>
+      <c r="L45" s="81"/>
     </row>
     <row r="46" spans="1:12" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="33">
         <v>21</v>
       </c>
       <c r="B46" s="34" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="C46" s="34"/>
-      <c r="D46" s="140"/>
-      <c r="E46" s="140"/>
-      <c r="F46" s="140"/>
-      <c r="G46" s="140"/>
-      <c r="H46" s="140"/>
-      <c r="I46" s="140"/>
-      <c r="J46" s="140"/>
-      <c r="K46" s="140"/>
-      <c r="L46" s="140"/>
+      <c r="D46" s="175"/>
+      <c r="E46" s="81"/>
+      <c r="F46" s="81"/>
+      <c r="G46" s="81"/>
+      <c r="H46" s="81"/>
+      <c r="I46" s="81"/>
+      <c r="J46" s="81"/>
+      <c r="K46" s="81"/>
+      <c r="L46" s="81"/>
     </row>
     <row r="47" spans="1:12" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="33">
         <v>22</v>
       </c>
       <c r="B47" s="34" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="C47" s="34"/>
-      <c r="D47" s="140"/>
-      <c r="E47" s="140"/>
-      <c r="F47" s="140"/>
-      <c r="G47" s="140"/>
-      <c r="H47" s="140"/>
-      <c r="I47" s="140"/>
-      <c r="J47" s="140"/>
-      <c r="K47" s="140"/>
-      <c r="L47" s="140"/>
+      <c r="D47" s="175"/>
+      <c r="E47" s="81"/>
+      <c r="F47" s="81"/>
+      <c r="G47" s="81"/>
+      <c r="H47" s="81"/>
+      <c r="I47" s="81"/>
+      <c r="J47" s="81"/>
+      <c r="K47" s="81"/>
+      <c r="L47" s="81"/>
     </row>
     <row r="48" spans="1:12" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="33">
         <v>23</v>
       </c>
       <c r="B48" s="34" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="C48" s="34"/>
-      <c r="D48" s="140"/>
-      <c r="E48" s="140"/>
-      <c r="F48" s="140"/>
-      <c r="G48" s="140"/>
-      <c r="H48" s="140"/>
-      <c r="I48" s="140"/>
-      <c r="J48" s="140"/>
-      <c r="K48" s="140"/>
-      <c r="L48" s="140"/>
+      <c r="D48" s="175"/>
+      <c r="E48" s="81"/>
+      <c r="F48" s="81"/>
+      <c r="G48" s="81"/>
+      <c r="H48" s="81"/>
+      <c r="I48" s="81"/>
+      <c r="J48" s="81"/>
+      <c r="K48" s="81"/>
+      <c r="L48" s="81"/>
     </row>
     <row r="49" spans="1:12" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="33">
         <v>24</v>
       </c>
       <c r="B49" s="34" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="C49" s="34"/>
-      <c r="D49" s="140"/>
-      <c r="E49" s="140"/>
-      <c r="F49" s="140"/>
-      <c r="G49" s="140"/>
-      <c r="H49" s="140"/>
-      <c r="I49" s="140"/>
-      <c r="J49" s="140"/>
-      <c r="K49" s="140"/>
-      <c r="L49" s="140"/>
+      <c r="D49" s="175"/>
+      <c r="E49" s="81"/>
+      <c r="F49" s="81"/>
+      <c r="G49" s="81"/>
+      <c r="H49" s="81"/>
+      <c r="I49" s="81"/>
+      <c r="J49" s="81"/>
+      <c r="K49" s="81"/>
+      <c r="L49" s="81"/>
     </row>
     <row r="50" spans="1:12" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="72">
         <v>25</v>
       </c>
       <c r="B50" s="77" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="C50" s="34"/>
-      <c r="D50" s="140"/>
-      <c r="E50" s="140"/>
-      <c r="F50" s="140"/>
-      <c r="G50" s="140"/>
-      <c r="H50" s="140"/>
-      <c r="I50" s="140"/>
-      <c r="J50" s="140"/>
-      <c r="K50" s="140"/>
-      <c r="L50" s="140"/>
+      <c r="D50" s="175"/>
+      <c r="E50" s="81"/>
+      <c r="F50" s="81"/>
+      <c r="G50" s="81"/>
+      <c r="H50" s="81"/>
+      <c r="I50" s="81"/>
+      <c r="J50" s="81"/>
+      <c r="K50" s="81"/>
+      <c r="L50" s="81"/>
     </row>
     <row r="51" spans="1:12" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="72">
         <v>26</v>
       </c>
       <c r="B51" s="77" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="C51" s="34"/>
-      <c r="D51" s="140"/>
-      <c r="E51" s="140"/>
-      <c r="F51" s="140"/>
-      <c r="G51" s="140"/>
-      <c r="H51" s="140"/>
-      <c r="I51" s="140"/>
-      <c r="J51" s="140"/>
-      <c r="K51" s="140"/>
-      <c r="L51" s="140"/>
+      <c r="D51" s="175"/>
+      <c r="E51" s="81"/>
+      <c r="F51" s="81"/>
+      <c r="G51" s="81"/>
+      <c r="H51" s="81"/>
+      <c r="I51" s="81"/>
+      <c r="J51" s="81"/>
+      <c r="K51" s="81"/>
+      <c r="L51" s="81"/>
     </row>
     <row r="52" spans="1:12" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="72">
         <v>27</v>
       </c>
       <c r="B52" s="77" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="C52" s="34"/>
-      <c r="D52" s="140"/>
-      <c r="E52" s="140"/>
-      <c r="F52" s="140"/>
-      <c r="G52" s="140"/>
-      <c r="H52" s="140"/>
-      <c r="I52" s="140"/>
-      <c r="J52" s="140"/>
-      <c r="K52" s="140"/>
-      <c r="L52" s="140"/>
+      <c r="D52" s="175"/>
+      <c r="E52" s="81"/>
+      <c r="F52" s="81"/>
+      <c r="G52" s="81"/>
+      <c r="H52" s="81"/>
+      <c r="I52" s="81"/>
+      <c r="J52" s="81"/>
+      <c r="K52" s="81"/>
+      <c r="L52" s="81"/>
     </row>
     <row r="53" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="72">
         <v>28</v>
       </c>
       <c r="B53" s="78" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C53" s="79"/>
-      <c r="D53" s="140"/>
-      <c r="E53" s="140"/>
-      <c r="F53" s="140"/>
-      <c r="G53" s="140"/>
-      <c r="H53" s="140"/>
-      <c r="I53" s="140"/>
-      <c r="J53" s="140"/>
-      <c r="K53" s="140"/>
-      <c r="L53" s="140"/>
+      <c r="D53" s="175"/>
+      <c r="E53" s="81"/>
+      <c r="F53" s="81"/>
+      <c r="G53" s="81"/>
+      <c r="H53" s="81"/>
+      <c r="I53" s="81"/>
+      <c r="J53" s="81"/>
+      <c r="K53" s="81"/>
+      <c r="L53" s="81"/>
     </row>
     <row r="54" spans="1:12" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="72">
@@ -12329,51 +12414,51 @@
         <v>144</v>
       </c>
       <c r="C54" s="72"/>
-      <c r="D54" s="140"/>
-      <c r="E54" s="140"/>
-      <c r="F54" s="140"/>
-      <c r="G54" s="140"/>
-      <c r="H54" s="140"/>
-      <c r="I54" s="140"/>
-      <c r="J54" s="140"/>
-      <c r="K54" s="140"/>
-      <c r="L54" s="140"/>
+      <c r="D54" s="175"/>
+      <c r="E54" s="81"/>
+      <c r="F54" s="81"/>
+      <c r="G54" s="81"/>
+      <c r="H54" s="81"/>
+      <c r="I54" s="81"/>
+      <c r="J54" s="81"/>
+      <c r="K54" s="81"/>
+      <c r="L54" s="81"/>
     </row>
     <row r="55" spans="1:12" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="72">
         <v>30</v>
       </c>
       <c r="B55" s="78" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C55" s="78"/>
-      <c r="D55" s="140"/>
-      <c r="E55" s="140"/>
-      <c r="F55" s="140"/>
-      <c r="G55" s="140"/>
-      <c r="H55" s="140"/>
-      <c r="I55" s="140"/>
-      <c r="J55" s="140"/>
-      <c r="K55" s="140"/>
-      <c r="L55" s="140"/>
+      <c r="D55" s="175"/>
+      <c r="E55" s="81"/>
+      <c r="F55" s="81"/>
+      <c r="G55" s="81"/>
+      <c r="H55" s="81"/>
+      <c r="I55" s="81"/>
+      <c r="J55" s="81"/>
+      <c r="K55" s="81"/>
+      <c r="L55" s="81"/>
     </row>
     <row r="56" spans="1:12" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="72">
         <v>31</v>
       </c>
       <c r="B56" s="78" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C56" s="78"/>
-      <c r="D56" s="140"/>
-      <c r="E56" s="140"/>
-      <c r="F56" s="140"/>
-      <c r="G56" s="140"/>
-      <c r="H56" s="140"/>
-      <c r="I56" s="140"/>
-      <c r="J56" s="140"/>
-      <c r="K56" s="140"/>
-      <c r="L56" s="140"/>
+      <c r="D56" s="175"/>
+      <c r="E56" s="81"/>
+      <c r="F56" s="81"/>
+      <c r="G56" s="81"/>
+      <c r="H56" s="81"/>
+      <c r="I56" s="81"/>
+      <c r="J56" s="81"/>
+      <c r="K56" s="81"/>
+      <c r="L56" s="81"/>
     </row>
     <row r="57" spans="1:12" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="72">
@@ -12383,26 +12468,36 @@
         <v>147</v>
       </c>
       <c r="C57" s="78"/>
-      <c r="D57" s="140"/>
-      <c r="E57" s="140"/>
-      <c r="F57" s="140"/>
-      <c r="G57" s="140"/>
-      <c r="H57" s="140"/>
-      <c r="I57" s="140"/>
-      <c r="J57" s="140"/>
-      <c r="K57" s="140"/>
-      <c r="L57" s="140"/>
+      <c r="D57" s="175"/>
+      <c r="E57" s="81"/>
+      <c r="F57" s="81"/>
+      <c r="G57" s="81"/>
+      <c r="H57" s="81"/>
+      <c r="I57" s="81"/>
+      <c r="J57" s="81"/>
+      <c r="K57" s="81"/>
+      <c r="L57" s="81"/>
+    </row>
+    <row r="58" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A58" s="173">
+        <v>33</v>
+      </c>
+      <c r="B58" s="78" t="s">
+        <v>148</v>
+      </c>
+      <c r="C58" s="78"/>
+      <c r="D58" s="175"/>
+      <c r="E58" s="81"/>
+      <c r="F58" s="81"/>
+      <c r="G58" s="81"/>
+      <c r="H58" s="81"/>
+      <c r="I58" s="81"/>
+      <c r="J58" s="81"/>
+      <c r="K58" s="81"/>
+      <c r="L58" s="81"/>
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="D26:L57"/>
-    <mergeCell ref="D18:D20"/>
-    <mergeCell ref="E18:L20"/>
-    <mergeCell ref="D25:L25"/>
-    <mergeCell ref="A23:L23"/>
-    <mergeCell ref="A24:L24"/>
-    <mergeCell ref="D21:D22"/>
-    <mergeCell ref="E21:L22"/>
     <mergeCell ref="A16:L16"/>
     <mergeCell ref="A17:L17"/>
     <mergeCell ref="B15:L15"/>
@@ -12414,6 +12509,14 @@
     <mergeCell ref="B4:L4"/>
     <mergeCell ref="B5:L5"/>
     <mergeCell ref="B7:L7"/>
+    <mergeCell ref="D18:D20"/>
+    <mergeCell ref="E18:L20"/>
+    <mergeCell ref="D25:L25"/>
+    <mergeCell ref="A23:L23"/>
+    <mergeCell ref="A24:L24"/>
+    <mergeCell ref="D21:D22"/>
+    <mergeCell ref="E21:L22"/>
+    <mergeCell ref="D26:L58"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="D26" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
@@ -15433,6 +15536,28 @@
                     <xdr:colOff>1409700</xdr:colOff>
                     <xdr:row>57</xdr:row>
                     <xdr:rowOff>7620</xdr:rowOff>
+                  </to>
+                </anchor>
+              </controlPr>
+            </control>
+          </mc:Choice>
+        </mc:AlternateContent>
+        <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+          <mc:Choice Requires="x14">
+            <control shapeId="1240" r:id="rId142" name="Drop Down 216">
+              <controlPr defaultSize="0" autoLine="0" autoPict="0">
+                <anchor moveWithCells="1">
+                  <from>
+                    <xdr:col>2</xdr:col>
+                    <xdr:colOff>0</xdr:colOff>
+                    <xdr:row>57</xdr:row>
+                    <xdr:rowOff>0</xdr:rowOff>
+                  </from>
+                  <to>
+                    <xdr:col>2</xdr:col>
+                    <xdr:colOff>1409700</xdr:colOff>
+                    <xdr:row>58</xdr:row>
+                    <xdr:rowOff>38100</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
@@ -15462,50 +15587,50 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="23.4" x14ac:dyDescent="0.3">
-      <c r="A1" s="150" t="s">
+      <c r="A1" s="149" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="151"/>
-      <c r="C1" s="151"/>
-      <c r="D1" s="151"/>
-      <c r="E1" s="151"/>
-      <c r="F1" s="151"/>
-      <c r="G1" s="151"/>
-      <c r="H1" s="151"/>
-      <c r="I1" s="151"/>
-      <c r="J1" s="151"/>
-      <c r="K1" s="151"/>
-      <c r="L1" s="152"/>
+      <c r="B1" s="150"/>
+      <c r="C1" s="150"/>
+      <c r="D1" s="150"/>
+      <c r="E1" s="150"/>
+      <c r="F1" s="150"/>
+      <c r="G1" s="150"/>
+      <c r="H1" s="150"/>
+      <c r="I1" s="150"/>
+      <c r="J1" s="150"/>
+      <c r="K1" s="150"/>
+      <c r="L1" s="151"/>
     </row>
     <row r="2" spans="1:12" ht="24" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="153" t="s">
+      <c r="A2" s="152" t="s">
         <v>40</v>
       </c>
-      <c r="B2" s="154"/>
-      <c r="C2" s="154"/>
-      <c r="D2" s="154"/>
-      <c r="E2" s="154"/>
-      <c r="F2" s="154"/>
-      <c r="G2" s="154"/>
-      <c r="H2" s="154"/>
-      <c r="I2" s="154"/>
-      <c r="J2" s="154"/>
-      <c r="K2" s="154"/>
-      <c r="L2" s="155"/>
+      <c r="B2" s="153"/>
+      <c r="C2" s="153"/>
+      <c r="D2" s="153"/>
+      <c r="E2" s="153"/>
+      <c r="F2" s="153"/>
+      <c r="G2" s="153"/>
+      <c r="H2" s="153"/>
+      <c r="I2" s="153"/>
+      <c r="J2" s="153"/>
+      <c r="K2" s="153"/>
+      <c r="L2" s="154"/>
     </row>
     <row r="3" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="156"/>
-      <c r="B3" s="157"/>
-      <c r="C3" s="157"/>
-      <c r="D3" s="157"/>
-      <c r="E3" s="157"/>
-      <c r="F3" s="157"/>
-      <c r="G3" s="157"/>
-      <c r="H3" s="157"/>
-      <c r="I3" s="157"/>
-      <c r="J3" s="157"/>
-      <c r="K3" s="157"/>
-      <c r="L3" s="158"/>
+      <c r="A3" s="155"/>
+      <c r="B3" s="156"/>
+      <c r="C3" s="156"/>
+      <c r="D3" s="156"/>
+      <c r="E3" s="156"/>
+      <c r="F3" s="156"/>
+      <c r="G3" s="156"/>
+      <c r="H3" s="156"/>
+      <c r="I3" s="156"/>
+      <c r="J3" s="156"/>
+      <c r="K3" s="156"/>
+      <c r="L3" s="157"/>
     </row>
     <row r="4" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A4" s="2"/>
@@ -15595,65 +15720,65 @@
       <c r="A8" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="B8" s="161"/>
-      <c r="C8" s="162"/>
-      <c r="D8" s="162"/>
-      <c r="E8" s="162"/>
-      <c r="F8" s="162"/>
-      <c r="G8" s="162"/>
-      <c r="H8" s="162"/>
-      <c r="I8" s="162"/>
-      <c r="J8" s="162"/>
-      <c r="K8" s="162"/>
-      <c r="L8" s="163"/>
+      <c r="B8" s="160"/>
+      <c r="C8" s="161"/>
+      <c r="D8" s="161"/>
+      <c r="E8" s="161"/>
+      <c r="F8" s="161"/>
+      <c r="G8" s="161"/>
+      <c r="H8" s="161"/>
+      <c r="I8" s="161"/>
+      <c r="J8" s="161"/>
+      <c r="K8" s="161"/>
+      <c r="L8" s="162"/>
     </row>
     <row r="9" spans="1:12" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="B9" s="164"/>
-      <c r="C9" s="162"/>
-      <c r="D9" s="162"/>
-      <c r="E9" s="162"/>
-      <c r="F9" s="162"/>
-      <c r="G9" s="162"/>
-      <c r="H9" s="162"/>
-      <c r="I9" s="162"/>
-      <c r="J9" s="162"/>
-      <c r="K9" s="162"/>
-      <c r="L9" s="163"/>
+      <c r="B9" s="163"/>
+      <c r="C9" s="161"/>
+      <c r="D9" s="161"/>
+      <c r="E9" s="161"/>
+      <c r="F9" s="161"/>
+      <c r="G9" s="161"/>
+      <c r="H9" s="161"/>
+      <c r="I9" s="161"/>
+      <c r="J9" s="161"/>
+      <c r="K9" s="161"/>
+      <c r="L9" s="162"/>
     </row>
     <row r="10" spans="1:12" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="159" t="s">
+      <c r="A10" s="158" t="s">
         <v>41</v>
       </c>
-      <c r="B10" s="160"/>
-      <c r="C10" s="160"/>
-      <c r="D10" s="160"/>
-      <c r="E10" s="160"/>
-      <c r="F10" s="160"/>
-      <c r="G10" s="160"/>
-      <c r="H10" s="160"/>
-      <c r="I10" s="160"/>
-      <c r="J10" s="160"/>
-      <c r="K10" s="160"/>
-      <c r="L10" s="160"/>
+      <c r="B10" s="159"/>
+      <c r="C10" s="159"/>
+      <c r="D10" s="159"/>
+      <c r="E10" s="159"/>
+      <c r="F10" s="159"/>
+      <c r="G10" s="159"/>
+      <c r="H10" s="159"/>
+      <c r="I10" s="159"/>
+      <c r="J10" s="159"/>
+      <c r="K10" s="159"/>
+      <c r="L10" s="159"/>
     </row>
     <row r="11" spans="1:12" ht="24" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="141" t="s">
+      <c r="A11" s="140" t="s">
         <v>34</v>
       </c>
-      <c r="B11" s="142"/>
-      <c r="C11" s="142"/>
-      <c r="D11" s="142"/>
-      <c r="E11" s="142"/>
-      <c r="F11" s="142"/>
-      <c r="G11" s="142"/>
-      <c r="H11" s="142"/>
-      <c r="I11" s="142"/>
-      <c r="J11" s="142"/>
-      <c r="K11" s="142"/>
-      <c r="L11" s="143"/>
+      <c r="B11" s="141"/>
+      <c r="C11" s="141"/>
+      <c r="D11" s="141"/>
+      <c r="E11" s="141"/>
+      <c r="F11" s="141"/>
+      <c r="G11" s="141"/>
+      <c r="H11" s="141"/>
+      <c r="I11" s="141"/>
+      <c r="J11" s="141"/>
+      <c r="K11" s="141"/>
+      <c r="L11" s="142"/>
     </row>
     <row r="12" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A12" s="16" t="s">
@@ -15665,101 +15790,101 @@
       <c r="C12" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="D12" s="123" t="s">
+      <c r="D12" s="90" t="s">
         <v>38</v>
       </c>
-      <c r="E12" s="123"/>
-      <c r="F12" s="123"/>
-      <c r="G12" s="123"/>
-      <c r="H12" s="123"/>
-      <c r="I12" s="123"/>
-      <c r="J12" s="123"/>
-      <c r="K12" s="123"/>
-      <c r="L12" s="123"/>
+      <c r="E12" s="90"/>
+      <c r="F12" s="90"/>
+      <c r="G12" s="90"/>
+      <c r="H12" s="90"/>
+      <c r="I12" s="90"/>
+      <c r="J12" s="90"/>
+      <c r="K12" s="90"/>
+      <c r="L12" s="90"/>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13" s="49"/>
       <c r="B13" s="50"/>
       <c r="C13" s="50"/>
-      <c r="D13" s="144"/>
-      <c r="E13" s="145"/>
-      <c r="F13" s="145"/>
-      <c r="G13" s="145"/>
-      <c r="H13" s="145"/>
-      <c r="I13" s="145"/>
-      <c r="J13" s="145"/>
-      <c r="K13" s="145"/>
-      <c r="L13" s="146"/>
+      <c r="D13" s="143"/>
+      <c r="E13" s="144"/>
+      <c r="F13" s="144"/>
+      <c r="G13" s="144"/>
+      <c r="H13" s="144"/>
+      <c r="I13" s="144"/>
+      <c r="J13" s="144"/>
+      <c r="K13" s="144"/>
+      <c r="L13" s="145"/>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14" s="49"/>
       <c r="B14" s="50"/>
       <c r="C14" s="50"/>
-      <c r="D14" s="147"/>
-      <c r="E14" s="148"/>
-      <c r="F14" s="148"/>
-      <c r="G14" s="148"/>
-      <c r="H14" s="148"/>
-      <c r="I14" s="148"/>
-      <c r="J14" s="148"/>
-      <c r="K14" s="148"/>
-      <c r="L14" s="149"/>
+      <c r="D14" s="146"/>
+      <c r="E14" s="147"/>
+      <c r="F14" s="147"/>
+      <c r="G14" s="147"/>
+      <c r="H14" s="147"/>
+      <c r="I14" s="147"/>
+      <c r="J14" s="147"/>
+      <c r="K14" s="147"/>
+      <c r="L14" s="148"/>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15" s="49"/>
       <c r="B15" s="50"/>
       <c r="C15" s="50"/>
-      <c r="D15" s="147"/>
-      <c r="E15" s="148"/>
-      <c r="F15" s="148"/>
-      <c r="G15" s="148"/>
-      <c r="H15" s="148"/>
-      <c r="I15" s="148"/>
-      <c r="J15" s="148"/>
-      <c r="K15" s="148"/>
-      <c r="L15" s="149"/>
+      <c r="D15" s="146"/>
+      <c r="E15" s="147"/>
+      <c r="F15" s="147"/>
+      <c r="G15" s="147"/>
+      <c r="H15" s="147"/>
+      <c r="I15" s="147"/>
+      <c r="J15" s="147"/>
+      <c r="K15" s="147"/>
+      <c r="L15" s="148"/>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A16" s="49"/>
       <c r="B16" s="50"/>
       <c r="C16" s="50"/>
-      <c r="D16" s="147"/>
-      <c r="E16" s="148"/>
-      <c r="F16" s="148"/>
-      <c r="G16" s="148"/>
-      <c r="H16" s="148"/>
-      <c r="I16" s="148"/>
-      <c r="J16" s="148"/>
-      <c r="K16" s="148"/>
-      <c r="L16" s="149"/>
+      <c r="D16" s="146"/>
+      <c r="E16" s="147"/>
+      <c r="F16" s="147"/>
+      <c r="G16" s="147"/>
+      <c r="H16" s="147"/>
+      <c r="I16" s="147"/>
+      <c r="J16" s="147"/>
+      <c r="K16" s="147"/>
+      <c r="L16" s="148"/>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A17" s="49"/>
       <c r="B17" s="50"/>
       <c r="C17" s="50"/>
-      <c r="D17" s="147"/>
-      <c r="E17" s="148"/>
-      <c r="F17" s="148"/>
-      <c r="G17" s="148"/>
-      <c r="H17" s="148"/>
-      <c r="I17" s="148"/>
-      <c r="J17" s="148"/>
-      <c r="K17" s="148"/>
-      <c r="L17" s="149"/>
+      <c r="D17" s="146"/>
+      <c r="E17" s="147"/>
+      <c r="F17" s="147"/>
+      <c r="G17" s="147"/>
+      <c r="H17" s="147"/>
+      <c r="I17" s="147"/>
+      <c r="J17" s="147"/>
+      <c r="K17" s="147"/>
+      <c r="L17" s="148"/>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A18" s="49"/>
       <c r="B18" s="50"/>
       <c r="C18" s="50"/>
-      <c r="D18" s="147"/>
-      <c r="E18" s="148"/>
-      <c r="F18" s="148"/>
-      <c r="G18" s="148"/>
-      <c r="H18" s="148"/>
-      <c r="I18" s="148"/>
-      <c r="J18" s="148"/>
-      <c r="K18" s="148"/>
-      <c r="L18" s="149"/>
+      <c r="D18" s="146"/>
+      <c r="E18" s="147"/>
+      <c r="F18" s="147"/>
+      <c r="G18" s="147"/>
+      <c r="H18" s="147"/>
+      <c r="I18" s="147"/>
+      <c r="J18" s="147"/>
+      <c r="K18" s="147"/>
+      <c r="L18" s="148"/>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -15848,10 +15973,10 @@
       <c r="B4" s="63"/>
     </row>
     <row r="6" spans="1:12" ht="18" x14ac:dyDescent="0.35">
-      <c r="A6" s="80" t="s">
+      <c r="A6" s="164" t="s">
         <v>42</v>
       </c>
-      <c r="B6" s="80"/>
+      <c r="B6" s="164"/>
     </row>
     <row r="8" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="66" t="s">
@@ -16583,6 +16708,68 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <SharedWithUsers xmlns="8029d101-3d2a-47c4-b15f-619642bf5e50">
+      <UserInfo>
+        <DisplayName>Luis Campos / Logiztik Alliance</DisplayName>
+        <AccountId>265</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Jairo Gonzalez / Logiztik Alliance</DisplayName>
+        <AccountId>322</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>José Ganchozo / Logiztik Alliance</DisplayName>
+        <AccountId>304</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Edwin Casa / Logiztik Alliance</DisplayName>
+        <AccountId>299</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Cristhian Cuichan / Logiztik Alliance</DisplayName>
+        <AccountId>369</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Oscar Yunda /  Logiztik Alliance</DisplayName>
+        <AccountId>355</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Fernando Ordoñez / Logiztik Alliance</DisplayName>
+        <AccountId>321</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Alex Rivera / Logiztik Alliance</DisplayName>
+        <AccountId>370</AccountId>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
+    <TaxCatchAll xmlns="8029d101-3d2a-47c4-b15f-619642bf5e50" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87481c51-c14c-4071-bf64-faa2b5708bb6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101005DA7AC6E4F4FAE42B9D9FCD9C82CAAE1" ma:contentTypeVersion="17" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="553e0bb76796fbad2df2b84fb95dc83d">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87481c51-c14c-4071-bf64-faa2b5708bb6" xmlns:ns3="8029d101-3d2a-47c4-b15f-619642bf5e50" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d87cd7f238c73dc12c577d08dde48736" ns2:_="" ns3:_="">
     <xsd:import namespace="87481c51-c14c-4071-bf64-faa2b5708bb6"/>
@@ -16831,69 +17018,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DD069904-634F-48DA-AA92-BAE250498BEE}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="8029d101-3d2a-47c4-b15f-619642bf5e50"/>
+    <ds:schemaRef ds:uri="87481c51-c14c-4071-bf64-faa2b5708bb6"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <SharedWithUsers xmlns="8029d101-3d2a-47c4-b15f-619642bf5e50">
-      <UserInfo>
-        <DisplayName>Luis Campos / Logiztik Alliance</DisplayName>
-        <AccountId>265</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Jairo Gonzalez / Logiztik Alliance</DisplayName>
-        <AccountId>322</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>José Ganchozo / Logiztik Alliance</DisplayName>
-        <AccountId>304</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Edwin Casa / Logiztik Alliance</DisplayName>
-        <AccountId>299</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Cristhian Cuichan / Logiztik Alliance</DisplayName>
-        <AccountId>369</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Oscar Yunda /  Logiztik Alliance</DisplayName>
-        <AccountId>355</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Fernando Ordoñez / Logiztik Alliance</DisplayName>
-        <AccountId>321</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Alex Rivera / Logiztik Alliance</DisplayName>
-        <AccountId>370</AccountId>
-        <AccountType/>
-      </UserInfo>
-    </SharedWithUsers>
-    <TaxCatchAll xmlns="8029d101-3d2a-47c4-b15f-619642bf5e50" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87481c51-c14c-4071-bf64-faa2b5708bb6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{371D8832-41B3-447B-B13D-2663C267E34F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2F7F06D0-41B3-4EAF-B418-88FC726117CC}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -16910,23 +17054,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{371D8832-41B3-447B-B13D-2663C267E34F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DD069904-634F-48DA-AA92-BAE250498BEE}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="8029d101-3d2a-47c4-b15f-619642bf5e50"/>
-    <ds:schemaRef ds:uri="87481c51-c14c-4071-bf64-faa2b5708bb6"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>